<commit_message>
Correct two labels in the All India downloads and the column glossary
women.csv: Bihar's district rows count the names removed in both phases,
and West Bengal's the fall from the 2024 roll to the 2026 election roll;
the measure column now says so. cities.csv: roll_before becomes base_roll,
with base_roll_is naming the roll, because Patna, Kolkata and Kochi are
measured on a different roll from the rest. The glossary now gives Bihar's
phase 2 total beside the Format 4B figure it differs from, and says where a
source does not record a date or a denominator. Workbooks and zip rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FWx24PCx3Jw4SUDQC6oU7o
</commit_message>
<xml_diff>
--- a/downloads/india-all-states.xlsx
+++ b/downloads/india-all-states.xlsx
@@ -1007,7 +1007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1015,11 +1015,12 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1050,25 +1051,30 @@
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>roll_before</t>
+          <t>base_roll</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
+          <t>base_roll_is</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
           <t>names_left_off_or_fall</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>per_100</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>state_per_100</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -1103,13 +1109,18 @@
       <c r="F2" t="n">
         <v>10388363</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
         <v>4688703</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>45.13</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>19.48</v>
       </c>
     </row>
@@ -1142,13 +1153,18 @@
       <c r="F3" t="n">
         <v>1851499</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
         <v>227324</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>12.28</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>19.48</v>
       </c>
     </row>
@@ -1181,13 +1197,18 @@
       <c r="F4" t="n">
         <v>43192452</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
         <v>5880312</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>13.61</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>19.48</v>
       </c>
     </row>
@@ -1220,16 +1241,21 @@
       <c r="F5" t="n">
         <v>4736669</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
         <v>1941444</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>40.99</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>21.7</v>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>figures as reported in the press</t>
         </is>
@@ -1264,16 +1290,21 @@
       <c r="F6" t="n">
         <v>8136309</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
         <v>2656935</v>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>32.66</v>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>21.7</v>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>figures as reported in the press</t>
         </is>
@@ -1308,16 +1339,21 @@
       <c r="F7" t="n">
         <v>20953470</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
         <v>2740856</v>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>13.08</v>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>21.7</v>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>figures as reported in the press</t>
         </is>
@@ -1352,13 +1388,18 @@
       <c r="F8" t="n">
         <v>4004694</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
         <v>1425018</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>35.58</v>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
         <v>15.19</v>
       </c>
     </row>
@@ -1391,13 +1432,18 @@
       <c r="F9" t="n">
         <v>7770786</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
         <v>1595922</v>
       </c>
-      <c r="H9" t="n">
+      <c r="I9" t="n">
         <v>20.54</v>
       </c>
-      <c r="I9" t="n">
+      <c r="J9" t="n">
         <v>15.19</v>
       </c>
     </row>
@@ -1430,13 +1476,18 @@
       <c r="F10" t="n">
         <v>52339107</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
         <v>6716891</v>
       </c>
-      <c r="H10" t="n">
+      <c r="I10" t="n">
         <v>12.83</v>
       </c>
-      <c r="I10" t="n">
+      <c r="J10" t="n">
         <v>15.19</v>
       </c>
     </row>
@@ -1469,13 +1520,18 @@
       <c r="F11" t="n">
         <v>10385510</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
         <v>3608922</v>
       </c>
-      <c r="H11" t="n">
+      <c r="I11" t="n">
         <v>34.75</v>
       </c>
-      <c r="I11" t="n">
+      <c r="J11" t="n">
         <v>21.14</v>
       </c>
     </row>
@@ -1508,13 +1564,18 @@
       <c r="F12" t="n">
         <v>9826568</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
         <v>3528086</v>
       </c>
-      <c r="H12" t="n">
+      <c r="I12" t="n">
         <v>35.9</v>
       </c>
-      <c r="I12" t="n">
+      <c r="J12" t="n">
         <v>21.14</v>
       </c>
     </row>
@@ -1547,13 +1608,18 @@
       <c r="F13" t="n">
         <v>77641971</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
         <v>13551479</v>
       </c>
-      <c r="H13" t="n">
+      <c r="I13" t="n">
         <v>17.45</v>
       </c>
-      <c r="I13" t="n">
+      <c r="J13" t="n">
         <v>21.14</v>
       </c>
     </row>
@@ -1586,13 +1652,18 @@
       <c r="F14" t="n">
         <v>9080173</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
         <v>2866481</v>
       </c>
-      <c r="H14" t="n">
+      <c r="I14" t="n">
         <v>31.57</v>
       </c>
-      <c r="I14" t="n">
+      <c r="J14" t="n">
         <v>21.14</v>
       </c>
     </row>
@@ -1625,13 +1696,18 @@
       <c r="F15" t="n">
         <v>88773876</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
         <v>17822006</v>
       </c>
-      <c r="H15" t="n">
+      <c r="I15" t="n">
         <v>20.08</v>
       </c>
-      <c r="I15" t="n">
+      <c r="J15" t="n">
         <v>21.14</v>
       </c>
     </row>
@@ -1664,15 +1740,20 @@
       <c r="F16" t="n">
         <v>14510299</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
         <v>4756722</v>
-      </c>
-      <c r="H16" t="n">
-        <v>32.78</v>
       </c>
       <c r="I16" t="n">
         <v>32.78</v>
       </c>
+      <c r="J16" t="n">
+        <v>32.78</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1703,13 +1784,18 @@
       <c r="F17" t="n">
         <v>4703664</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
         <v>1265610</v>
       </c>
-      <c r="H17" t="n">
+      <c r="I17" t="n">
         <v>26.91</v>
       </c>
-      <c r="I17" t="n">
+      <c r="J17" t="n">
         <v>32.78</v>
       </c>
     </row>
@@ -1742,13 +1828,18 @@
       <c r="F18" t="n">
         <v>3994535</v>
       </c>
-      <c r="G18" t="n">
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
         <v>1200138</v>
       </c>
-      <c r="H18" t="n">
+      <c r="I18" t="n">
         <v>30.04</v>
       </c>
-      <c r="I18" t="n">
+      <c r="J18" t="n">
         <v>18.7</v>
       </c>
     </row>
@@ -1781,13 +1872,18 @@
       <c r="F19" t="n">
         <v>4656702</v>
       </c>
-      <c r="G19" t="n">
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
         <v>780325</v>
       </c>
-      <c r="H19" t="n">
+      <c r="I19" t="n">
         <v>16.76</v>
       </c>
-      <c r="I19" t="n">
+      <c r="J19" t="n">
         <v>18.7</v>
       </c>
     </row>
@@ -1820,13 +1916,18 @@
       <c r="F20" t="n">
         <v>145778855</v>
       </c>
-      <c r="G20" t="n">
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
         <v>26893604</v>
       </c>
-      <c r="H20" t="n">
+      <c r="I20" t="n">
         <v>18.45</v>
       </c>
-      <c r="I20" t="n">
+      <c r="J20" t="n">
         <v>18.7</v>
       </c>
     </row>
@@ -1859,13 +1960,18 @@
       <c r="F21" t="n">
         <v>6259620</v>
       </c>
-      <c r="G21" t="n">
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
         <v>1452704</v>
       </c>
-      <c r="H21" t="n">
+      <c r="I21" t="n">
         <v>23.21</v>
       </c>
-      <c r="I21" t="n">
+      <c r="J21" t="n">
         <v>14.5</v>
       </c>
     </row>
@@ -1898,13 +2004,18 @@
       <c r="F22" t="n">
         <v>1389712</v>
       </c>
-      <c r="G22" t="n">
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
         <v>215786</v>
       </c>
-      <c r="H22" t="n">
+      <c r="I22" t="n">
         <v>15.53</v>
       </c>
-      <c r="I22" t="n">
+      <c r="J22" t="n">
         <v>14.5</v>
       </c>
     </row>
@@ -1937,13 +2048,18 @@
       <c r="F23" t="n">
         <v>43194104</v>
       </c>
-      <c r="G23" t="n">
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
         <v>5704837</v>
       </c>
-      <c r="H23" t="n">
+      <c r="I23" t="n">
         <v>13.21</v>
       </c>
-      <c r="I23" t="n">
+      <c r="J23" t="n">
         <v>14.5</v>
       </c>
     </row>
@@ -1976,13 +2092,18 @@
       <c r="F24" t="n">
         <v>4873512</v>
       </c>
-      <c r="G24" t="n">
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
         <v>1250319</v>
       </c>
-      <c r="H24" t="n">
+      <c r="I24" t="n">
         <v>25.66</v>
       </c>
-      <c r="I24" t="n">
+      <c r="J24" t="n">
         <v>14.5</v>
       </c>
     </row>
@@ -2015,13 +2136,18 @@
       <c r="F25" t="n">
         <v>45969924</v>
       </c>
-      <c r="G25" t="n">
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>roll before the revision</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
         <v>6123008</v>
       </c>
-      <c r="H25" t="n">
+      <c r="I25" t="n">
         <v>13.32</v>
       </c>
-      <c r="I25" t="n">
+      <c r="J25" t="n">
         <v>14.5</v>
       </c>
     </row>
@@ -2054,16 +2180,21 @@
       <c r="F26" t="n">
         <v>4843590</v>
       </c>
-      <c r="G26" t="n">
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2025 election roll</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
         <v>415580</v>
       </c>
-      <c r="H26" t="n">
+      <c r="I26" t="n">
         <v>8.58</v>
       </c>
-      <c r="I26" t="n">
+      <c r="J26" t="n">
         <v>9.25</v>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>per 100 on the 2025 roll</t>
         </is>
@@ -2098,16 +2229,21 @@
       <c r="F27" t="n">
         <v>69856324</v>
       </c>
-      <c r="G27" t="n">
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2025 election roll</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
         <v>6494979</v>
       </c>
-      <c r="H27" t="n">
+      <c r="I27" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="I27" t="n">
+      <c r="J27" t="n">
         <v>9.25</v>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>per 100 on the 2025 roll</t>
         </is>
@@ -2142,13 +2278,18 @@
       <c r="F28" t="n">
         <v>2405408</v>
       </c>
-      <c r="G28" t="n">
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2024 Lok Sabha roll</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
         <v>598153</v>
       </c>
-      <c r="H28" t="n">
+      <c r="I28" t="n">
         <v>24.87</v>
       </c>
-      <c r="I28" t="n">
+      <c r="J28" t="n">
         <v>6.83</v>
       </c>
     </row>
@@ -2181,13 +2322,18 @@
       <c r="F29" t="n">
         <v>12360295</v>
       </c>
-      <c r="G29" t="n">
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2024 Lok Sabha roll</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
         <v>1158176</v>
       </c>
-      <c r="H29" t="n">
+      <c r="I29" t="n">
         <v>9.369999999999999</v>
       </c>
-      <c r="I29" t="n">
+      <c r="J29" t="n">
         <v>6.83</v>
       </c>
     </row>
@@ -2220,13 +2366,18 @@
       <c r="F30" t="n">
         <v>61244303</v>
       </c>
-      <c r="G30" t="n">
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2024 Lok Sabha roll</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
         <v>3437047</v>
       </c>
-      <c r="H30" t="n">
+      <c r="I30" t="n">
         <v>5.61</v>
       </c>
-      <c r="I30" t="n">
+      <c r="J30" t="n">
         <v>6.83</v>
       </c>
     </row>
@@ -2259,13 +2410,18 @@
       <c r="F31" t="n">
         <v>2638106</v>
       </c>
-      <c r="G31" t="n">
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>January 2025 roll</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
         <v>307463</v>
       </c>
-      <c r="H31" t="n">
+      <c r="I31" t="n">
         <v>11.65</v>
       </c>
-      <c r="I31" t="n">
+      <c r="J31" t="n">
         <v>8.52</v>
       </c>
     </row>
@@ -2298,13 +2454,18 @@
       <c r="F32" t="n">
         <v>25172836</v>
       </c>
-      <c r="G32" t="n">
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>January 2025 roll</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
         <v>2061127</v>
       </c>
-      <c r="H32" t="n">
+      <c r="I32" t="n">
         <v>8.19</v>
       </c>
-      <c r="I32" t="n">
+      <c r="J32" t="n">
         <v>8.52</v>
       </c>
     </row>
@@ -4743,7 +4904,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -4774,7 +4935,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -4805,7 +4966,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -4836,7 +4997,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -4867,7 +5028,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -4898,7 +5059,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -4929,7 +5090,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -4960,7 +5121,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -4991,7 +5152,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -5022,7 +5183,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -5053,7 +5214,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -5084,7 +5245,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -5115,7 +5276,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -5146,7 +5307,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -5177,7 +5338,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -5208,7 +5369,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -5239,7 +5400,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -5270,7 +5431,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -5301,7 +5462,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -5332,7 +5493,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -5363,7 +5524,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -5394,7 +5555,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -5425,7 +5586,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -5456,7 +5617,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -5487,7 +5648,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -5518,7 +5679,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -5549,7 +5710,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E39" t="n">
@@ -5580,7 +5741,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -5611,7 +5772,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -5642,7 +5803,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -5673,7 +5834,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -5704,7 +5865,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -5735,7 +5896,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -5766,7 +5927,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -5797,7 +5958,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -5828,7 +5989,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -5859,7 +6020,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -5890,7 +6051,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>names removed at the draft</t>
+          <t>names removed in both phases</t>
         </is>
       </c>
       <c r="E50" t="n">
@@ -5921,7 +6082,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E51" t="n">
@@ -5952,7 +6113,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E52" t="n">
@@ -5983,7 +6144,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E53" t="n">
@@ -6014,7 +6175,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E54" t="n">
@@ -6045,7 +6206,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E55" t="n">
@@ -6076,7 +6237,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E56" t="n">
@@ -6107,7 +6268,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E57" t="n">
@@ -6138,7 +6299,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -6169,7 +6330,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E59" t="n">
@@ -6200,7 +6361,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -6231,7 +6392,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E61" t="n">
@@ -6262,7 +6423,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E62" t="n">
@@ -6293,7 +6454,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E63" t="n">
@@ -6324,7 +6485,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E64" t="n">
@@ -6355,7 +6516,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E65" t="n">
@@ -6386,7 +6547,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -6417,7 +6578,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E67" t="n">
@@ -6448,7 +6609,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E68" t="n">
@@ -6479,7 +6640,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E69" t="n">
@@ -6510,7 +6671,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -6541,7 +6702,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E71" t="n">
@@ -6572,7 +6733,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -6603,7 +6764,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E73" t="n">
@@ -6634,7 +6795,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>fall in the roll, 2024 roll to the draft</t>
+          <t>fall in the roll, 2024 roll to the 2026 election roll</t>
         </is>
       </c>
       <c r="E74" t="n">
@@ -47755,7 +47916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C184"/>
+  <dimension ref="A1:C185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -48473,7 +48634,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>People born in the state and counted living in another state at the 2011 census, as a percentage, from the census place-of-birth tables.</t>
+          <t>People born in the state and counted living in another state at the 2011 census, as a percentage, from Census table D-01 (place of birth). The curated file does not record which population the percentage is of.</t>
         </is>
       </c>
     </row>
@@ -48490,7 +48651,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>People counted living in the state at the 2011 census who were born in another state, as a percentage, from the census place-of-birth tables.</t>
+          <t>People counted living in the state at the 2011 census who were born in another state, as a percentage, from Census table D-01 (place of birth). The curated file does not record which population the percentage is of.</t>
         </is>
       </c>
     </row>
@@ -49930,12 +50091,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>roll_before</t>
+          <t>base_roll</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Electors on the roll the count is measured against, as a count, which is the roll before the revision except for Patna (the 2025 roll), Kolkata (the 2024 Lok Sabha roll) and Kochi (the January 2025 roll).</t>
+          <t>Electors on the roll the count is measured against, the roll named in base_roll_is.</t>
         </is>
       </c>
     </row>
@@ -49947,12 +50108,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>names_left_off_or_fall</t>
+          <t>base_roll_is</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Names left off the draft, or for Kolkata and Kochi the fall in the roll to the draft, as a count (Patna counts both of Bihar's phases).</t>
+          <t>Which roll base_roll is. It is the roll before the revision everywhere except Patna (the 2025 election roll), Kolkata (the 2024 Lok Sabha roll) and Kochi (the January 2025 roll).</t>
         </is>
       </c>
     </row>
@@ -49964,12 +50125,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>per_100</t>
+          <t>names_left_off_or_fall</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>names_left_off_or_fall per 100 electors on roll_before.</t>
+          <t>Names left off the draft, or for Kolkata and Kochi the fall in the roll to the draft, as a count (Patna counts both of Bihar's phases).</t>
         </is>
       </c>
     </row>
@@ -49981,12 +50142,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>state_per_100</t>
+          <t>per_100</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>The same rate for the city's whole state.</t>
+          <t>names_left_off_or_fall per 100 electors on roll_before.</t>
         </is>
       </c>
     </row>
@@ -49998,29 +50159,29 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>state_per_100</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>A note where the row's figures differ in kind, marking Hyderabad's figures as reported in the press and Patna's as per 100 on the 2025 roll.</t>
+          <t>The same rate for the city's whole state.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Reserved and general seats</t>
+          <t>Cities against their states</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>note</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>The state.</t>
+          <t>A note where the row's figures differ in kind, marking Hyderabad's figures as reported in the press and Patna's as per 100 on the 2025 roll.</t>
         </is>
       </c>
     </row>
@@ -50032,12 +50193,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>measure</t>
+          <t>state</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>The count and its base, which is names removed in both phases per 100 on the 2025 roll for Bihar, names left off per 100 on the roll before for Tamil Nadu, Gujarat and Delhi, and the fall in the roll to the draft per 100 for West Bengal (from the 2024 roll) and Kerala (from the January 2025 roll).</t>
+          <t>The state.</t>
         </is>
       </c>
     </row>
@@ -50049,12 +50210,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>measure</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>The kind of seat under the Delimitation Order of 2008, GEN for general, SC for Scheduled Castes and ST for Scheduled Tribes.</t>
+          <t>The count and its base, which is names removed in both phases per 100 on the 2025 roll for Bihar, names left off per 100 on the roll before for Tamil Nadu, Gujarat and Delhi, and the fall in the roll to the draft per 100 for West Bengal (from the 2024 roll) and Kerala (from the January 2025 roll).</t>
         </is>
       </c>
     </row>
@@ -50066,12 +50227,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>seats</t>
+          <t>category</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>The number of assembly seats in that category.</t>
+          <t>The kind of seat under the Delimitation Order of 2008, GEN for general, SC for Scheduled Castes and ST for Scheduled Tribes.</t>
         </is>
       </c>
     </row>
@@ -50083,12 +50244,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>rate</t>
+          <t>seats</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>The count per 100 electors across all seats in the category, in the measure named.</t>
+          <t>The number of assembly seats in that category.</t>
         </is>
       </c>
     </row>
@@ -50100,12 +50261,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>mean_gap_vs_general_seats_same_district</t>
+          <t>rate</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>The average, over the reserved seats, of each seat's rate less the rate of the general seats in its own district, in points per 100, blank for general seats.</t>
+          <t>The count per 100 electors across all seats in the category, in the measure named.</t>
         </is>
       </c>
     </row>
@@ -50117,12 +50278,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>seats_above_their_district</t>
+          <t>mean_gap_vs_general_seats_same_district</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>How many reserved seats have a higher rate than the general seats of their own district.</t>
+          <t>The average, over the reserved seats, of each seat's rate less the rate of the general seats in its own district, in points per 100, blank for general seats.</t>
         </is>
       </c>
     </row>
@@ -50134,29 +50295,29 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>seats_compared</t>
+          <t>seats_above_their_district</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>How many reserved seats had general seats in their district to be compared with.</t>
+          <t>How many reserved seats have a higher rate than the general seats of their own district.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Border districts against the re</t>
+          <t>Reserved and general seats</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>seats_compared</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>The state.</t>
+          <t>How many reserved seats had general seats in their district to be compared with.</t>
         </is>
       </c>
     </row>
@@ -50168,12 +50329,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>measure</t>
+          <t>state</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>The count and its base, which is names left off per 100 on the roll before (Uttar Pradesh, Gujarat), names removed in both phases per 100 on the 2025 roll (Bihar), the fall in the roll per 100 from the 2024 roll to the draft (West Bengal) and names removed after the draft per 1,000 on the draft (Uttarakhand).</t>
+          <t>The state.</t>
         </is>
       </c>
     </row>
@@ -50185,12 +50346,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>part</t>
+          <t>measure</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Which districts the row covers, where border is every district on the Government of India's list of Border Guarding Districts, interior the rest, interior_without_city the rest without the city's districts, and border district names one listed district.</t>
+          <t>The count and its base, which is names left off per 100 on the roll before (Uttar Pradesh, Gujarat), names removed in both phases per 100 on the 2025 roll (Bihar), the fall in the roll per 100 from the 2024 roll to the draft (West Bengal) and names removed after the draft per 1,000 on the draft (Uttarakhand).</t>
         </is>
       </c>
     </row>
@@ -50202,12 +50363,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>districts</t>
+          <t>part</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>The number of districts in the row.</t>
+          <t>Which districts the row covers, where border is every district on the Government of India's list of Border Guarding Districts, interior the rest, interior_without_city the rest without the city's districts, and border district names one listed district.</t>
         </is>
       </c>
     </row>
@@ -50219,12 +50380,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>districts</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Electors on the roll the measure divides by, summed over the districts, blank on single-district rows.</t>
+          <t>The number of districts in the row.</t>
         </is>
       </c>
     </row>
@@ -50236,12 +50397,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>base</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>The count the measure names, summed over the districts, blank on single-district rows.</t>
+          <t>Electors on the roll the measure divides by, summed over the districts, blank on single-district rows.</t>
         </is>
       </c>
     </row>
@@ -50253,12 +50414,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>rate</t>
+          <t>count</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>count per 100 electors on base, or per 1,000 for Uttarakhand.</t>
+          <t>The count the measure names, summed over the districts, blank on single-district rows.</t>
         </is>
       </c>
     </row>
@@ -50270,12 +50431,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>dead_share</t>
+          <t>rate</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>The share of the count entered as dead, as a percentage, where reasons were published (Uttar Pradesh and Gujarat), and the reason is what the officer wrote down, and nobody checked it.</t>
+          <t>count per 100 electors on base, or per 1,000 for Uttarakhand.</t>
         </is>
       </c>
     </row>
@@ -50287,12 +50448,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>shifted_absent_share</t>
+          <t>dead_share</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>The share of the count entered as shifted or absent, as a percentage, where reasons were published.</t>
+          <t>The share of the count entered as dead, as a percentage, where reasons were published (Uttar Pradesh and Gujarat), and the reason is what the officer wrote down, and nobody checked it.</t>
         </is>
       </c>
     </row>
@@ -50304,29 +50465,29 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>enrolled_elsewhere_share</t>
+          <t>shifted_absent_share</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>The share of the count entered as enrolled somewhere else, as a percentage, where reasons were published.</t>
+          <t>The share of the count entered as shifted or absent, as a percentage, where reasons were published.</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Women, state by state and distr</t>
+          <t>Border districts against the re</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>enrolled_elsewhere_share</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Whether the row is a whole state or one district.</t>
+          <t>The share of the count entered as enrolled somewhere else, as a percentage, where reasons were published.</t>
         </is>
       </c>
     </row>
@@ -50338,12 +50499,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>level</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>The state.</t>
+          <t>Whether the row is a whole state or one district.</t>
         </is>
       </c>
     </row>
@@ -50355,12 +50516,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>state</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>The district, blank on state rows.</t>
+          <t>The state.</t>
         </is>
       </c>
     </row>
@@ -50372,12 +50533,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>measure</t>
+          <t>district</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>The count the row's shares are of, as labelled by the build, and for West Bengal's district rows the share is in fact of the fall to the 2026 election roll while for Bihar's it is of the names removed in both phases.</t>
+          <t>The district, blank on state rows.</t>
         </is>
       </c>
     </row>
@@ -50389,12 +50550,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>women_share_of_roll</t>
+          <t>measure</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Women as a percentage of the roll the count is taken from (the roll before for states, Bihar's draft plus phase 1 removals, the 2024 and January 2025 rolls for West Bengal and Kerala, and the draft for Uttarakhand).</t>
+          <t>The count the row's shares are of. For district rows it names the state's own measure, such as the names removed in both phases in Bihar or the fall from the 2024 roll to the 2026 election roll in West Bengal.</t>
         </is>
       </c>
     </row>
@@ -50406,12 +50567,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>women_share_of_count</t>
+          <t>women_share_of_roll</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Women as a percentage of the count named in measure.</t>
+          <t>Women as a percentage of the roll the count is taken from (the roll before for states, Bihar's draft plus phase 1 removals, the 2024 and January 2025 rolls for West Bengal and Kerala, and the draft for Uttarakhand).</t>
         </is>
       </c>
     </row>
@@ -50423,12 +50584,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>gap_points</t>
+          <t>women_share_of_count</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>women_share_of_count less women_share_of_roll, in percentage points.</t>
+          <t>Women as a percentage of the count named in measure.</t>
         </is>
       </c>
     </row>
@@ -50440,12 +50601,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>women_left_off_per_100_women</t>
+          <t>gap_points</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Women left off the draft per 100 women on the roll before, where the roll by sex is the roll before times women's share of it, on state rows only.</t>
+          <t>women_share_of_count less women_share_of_roll, in percentage points.</t>
         </is>
       </c>
     </row>
@@ -50457,12 +50618,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>men_left_off_per_100_men</t>
+          <t>women_left_off_per_100_women</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Men left off the draft per 100 men on the roll before, on state rows only.</t>
+          <t>Women left off the draft per 100 women on the roll before, where the roll by sex is the roll before times women's share of it, on state rows only.</t>
         </is>
       </c>
     </row>
@@ -50474,12 +50635,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>quality</t>
+          <t>men_left_off_per_100_men</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>How firm the state's split by sex is (lists, exact, rounded, proxy or unverified), on state rows only.</t>
+          <t>Men left off the draft per 100 men on the roll before, on state rows only.</t>
         </is>
       </c>
     </row>
@@ -50491,29 +50652,29 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>source_url</t>
+          <t>quality</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>The address of the source of the state's split by sex, on state rows only.</t>
+          <t>How firm the state's split by sex is (lists, exact, rounded, proxy or unverified), on state rows only.</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Rural, mixed and urban district</t>
+          <t>Women, state by state and distr</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>source_url</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>The state.</t>
+          <t>The address of the source of the state's split by sex, on state rows only.</t>
         </is>
       </c>
     </row>
@@ -50525,12 +50686,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>measure</t>
+          <t>state</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>What is counted, where left_off means names left off the draft per 100 on the roll before, roll_2025 means Bihar's names removed in both phases per 100 on the 2025 roll, and fall means the fall in the roll to the draft (West Bengal from the 2024 roll, Kerala from the January 2025 roll).</t>
+          <t>The state.</t>
         </is>
       </c>
     </row>
@@ -50542,12 +50703,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>district_2011</t>
+          <t>measure</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>The district as it stood at the 2011 census, which is the unit each row adds up.</t>
+          <t>What is counted, where left_off means names left off the draft per 100 on the roll before, roll_2025 means Bihar's names removed in both phases per 100 on the 2025 roll, and fall means the fall in the roll to the draft (West Bengal from the 2024 roll, Kerala from the January 2025 roll).</t>
         </is>
       </c>
     </row>
@@ -50559,12 +50720,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>census_code</t>
+          <t>district_2011</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>The 2011 census code of that district.</t>
+          <t>The district as it stood at the 2011 census, which is the unit each row adds up.</t>
         </is>
       </c>
     </row>
@@ -50576,12 +50737,12 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>districts_today</t>
+          <t>census_code</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>The present districts counted under it, each under the 2011 district it was mostly made from, separated by a semicolon character.</t>
+          <t>The 2011 census code of that district.</t>
         </is>
       </c>
     </row>
@@ -50593,12 +50754,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>urban_pct_2011</t>
+          <t>districts_today</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>The share of the 2011 district's people living in towns at the 2011 census, as a percentage, from table A-01.</t>
+          <t>The present districts counted under it, each under the 2011 district it was mostly made from, separated by a semicolon character.</t>
         </is>
       </c>
     </row>
@@ -50610,12 +50771,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>band</t>
+          <t>urban_pct_2011</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>rural where urban_pct_2011 is under 20, mixed from 20 to 50, and urban above 50.</t>
+          <t>The share of the 2011 district's people living in towns at the 2011 census, as a percentage, from table A-01.</t>
         </is>
       </c>
     </row>
@@ -50627,12 +50788,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>roll_before</t>
+          <t>band</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Electors on the roll the count is measured against, summed over the districts, as a count.</t>
+          <t>rural where urban_pct_2011 is under 20, mixed from 20 to 50, and urban above 50.</t>
         </is>
       </c>
     </row>
@@ -50644,12 +50805,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>roll_before</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Names left off, or the fall in the roll, summed over the districts, as a count.</t>
+          <t>Electors on the roll the count is measured against, summed over the districts, as a count.</t>
         </is>
       </c>
     </row>
@@ -50661,29 +50822,29 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>per_100</t>
+          <t>count</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>count per 100 electors on roll_before.</t>
+          <t>Names left off, or the fall in the roll, summed over the districts, as a count.</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>Rural, mixed and urban district</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>per_100</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>The state, one of the four that published their rolls by constituency (Tamil Nadu, Kerala, West Bengal and Uttarakhand).</t>
+          <t>count per 100 electors on roll_before.</t>
         </is>
       </c>
     </row>
@@ -50695,12 +50856,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>ac</t>
+          <t>state</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>The assembly constituency number.</t>
+          <t>The state, one of the four that published their rolls by constituency (Tamil Nadu, Kerala, West Bengal and Uttarakhand).</t>
         </is>
       </c>
     </row>
@@ -50712,12 +50873,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>constituency</t>
+          <t>ac</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>The assembly constituency's name.</t>
+          <t>The assembly constituency number.</t>
         </is>
       </c>
     </row>
@@ -50729,12 +50890,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>constituency</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>The district the constituency lies in.</t>
+          <t>The assembly constituency's name.</t>
         </is>
       </c>
     </row>
@@ -50746,12 +50907,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>earlier_roll</t>
+          <t>district</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>The earliest roll in the row, which is the roll of 27 October 2025 worked out as the draft plus the names left off for Tamil Nadu, the January 2025 final roll for Kerala, the 2024 Lok Sabha roll for West Bengal and blank for Uttarakhand.</t>
+          <t>The district the constituency lies in.</t>
         </is>
       </c>
     </row>
@@ -50763,12 +50924,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>left_off_draft</t>
+          <t>earlier_roll</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Names left off the draft, as a count, given by constituency only in Tamil Nadu.</t>
+          <t>The earliest roll in the row, which is the roll of 27 October 2025 worked out as the draft plus the names left off for Tamil Nadu, the January 2025 final roll for Kerala, the 2024 Lok Sabha roll for West Bengal and blank for Uttarakhand.</t>
         </is>
       </c>
     </row>
@@ -50780,12 +50941,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>left_off_draft</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Electors on the draft roll (19 December 2025 in Tamil Nadu, 23 December 2025 in Kerala, 16 December 2025 in West Bengal, July 2026 in Uttarakhand).</t>
+          <t>Names left off the draft, as a count, given by constituency only in Tamil Nadu.</t>
         </is>
       </c>
     </row>
@@ -50797,12 +50958,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>added_after_draft</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Claims admitted after the draft, as a count, Uttarakhand only, from the Chief Electoral Officer's PN 63/2026.</t>
+          <t>Electors on the draft roll (19 December 2025 in Tamil Nadu, 23 December 2025 in Kerala, 16 December 2025 in West Bengal, July 2026 in Uttarakhand).</t>
         </is>
       </c>
     </row>
@@ -50814,12 +50975,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>removed_after_draft</t>
+          <t>added_after_draft</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Objections admitted after the draft, as a count, Uttarakhand only, from PN 63/2026.</t>
+          <t>Claims admitted after the draft, as a count, Uttarakhand only, from the Chief Electoral Officer's PN 63/2026.</t>
         </is>
       </c>
     </row>
@@ -50831,12 +50992,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>later_roll</t>
+          <t>removed_after_draft</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>The latest roll in the row, the final roll of 23 February 2026 in Tamil Nadu, 21 February 2026 in Kerala and 3 October 2026 in Uttarakhand, and the roll at the 2026 nominations in West Bengal.</t>
+          <t>Objections admitted after the draft, as a count, Uttarakhand only, from PN 63/2026.</t>
         </is>
       </c>
     </row>
@@ -50848,12 +51009,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>change_draft_to_later</t>
+          <t>later_roll</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>later_roll less draft, a net change that counts new voters added after the draft as well as names put back.</t>
+          <t>The latest roll in the row, the final roll of 23 February 2026 in Tamil Nadu, 21 February 2026 in Kerala and 3 October 2026 in Uttarakhand, and the roll at the 2026 nominations in West Bengal.</t>
         </is>
       </c>
     </row>
@@ -50865,12 +51026,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>change_earlier_to_later</t>
+          <t>change_draft_to_later</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>later_roll less earlier_roll, as a count, which is negative where the roll fell.</t>
+          <t>later_roll less draft, a net change that counts new voters added after the draft as well as names put back.</t>
         </is>
       </c>
     </row>
@@ -50882,10 +51043,27 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
+          <t>change_earlier_to_later</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>later_roll less earlier_roll, as a count, which is negative where the roll fell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
           <t>change_earlier_to_later_per_100</t>
         </is>
       </c>
-      <c r="C184" t="inlineStr">
+      <c r="C185" t="inlineStr">
         <is>
           <t>change_earlier_to_later per 100 electors on earlier_roll.</t>
         </is>

</xml_diff>

<commit_message>
Bihar electors from the Commission's results; migration denominator settled from Census D-01
Bihar's 2025 electors now come from the Election Commission's Detailed
Results rather than the Wikipedia seat list, which carried slips in five
seats (Bahadurpur by 9,000, Bahadurganj by 1,100). Rates move in those five
seats; the over-margin counts and the swing slope are unchanged, and the
thirds of seats now show the NDA's lead growing 4.5 to 4.7 points.
verify_bihar.py reads the same source. Reports and decks rebuilt.

Census D-01 shows both migration shares are counts over the state's own 2011
population; the extract is in data/india/raw/census2011_d01_states.csv and
check_data.py now holds covariates.csv to it.

The glossary records what the research found on Bihar's phase 2 count and
the Hyderabad base roll.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FWx24PCx3Jw4SUDQC6oU7o
</commit_message>
<xml_diff>
--- a/downloads/india-all-states.xlsx
+++ b/downloads/india-all-states.xlsx
@@ -2227,7 +2227,7 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>69856324</v>
+        <v>69846731</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -3581,7 +3581,7 @@
         <v>7</v>
       </c>
       <c r="E18" t="n">
-        <v>16316534</v>
+        <v>16314914</v>
       </c>
       <c r="F18" t="n">
         <v>1624329</v>
@@ -3610,13 +3610,13 @@
         <v>31</v>
       </c>
       <c r="E19" t="n">
-        <v>58383380</v>
+        <v>58375407</v>
       </c>
       <c r="F19" t="n">
         <v>5286230</v>
       </c>
       <c r="G19" t="n">
-        <v>9.050000000000001</v>
+        <v>9.06</v>
       </c>
     </row>
     <row r="20">
@@ -3639,7 +3639,7 @@
         <v>30</v>
       </c>
       <c r="E20" t="n">
-        <v>53539790</v>
+        <v>53531817</v>
       </c>
       <c r="F20" t="n">
         <v>4870650</v>
@@ -3668,7 +3668,7 @@
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>13.9</v>
+        <v>13.92</v>
       </c>
     </row>
     <row r="22">
@@ -17164,13 +17164,13 @@
         </is>
       </c>
       <c r="H226" t="n">
-        <v>1127532</v>
+        <v>1125912</v>
       </c>
       <c r="I226" t="n">
         <v>156727</v>
       </c>
       <c r="J226" t="n">
-        <v>13.9</v>
+        <v>13.92</v>
       </c>
     </row>
     <row r="227">
@@ -17290,13 +17290,13 @@
         </is>
       </c>
       <c r="H229" t="n">
-        <v>2902355</v>
+        <v>2894382</v>
       </c>
       <c r="I229" t="n">
         <v>210711</v>
       </c>
       <c r="J229" t="n">
-        <v>7.26</v>
+        <v>7.28</v>
       </c>
     </row>
     <row r="230">
@@ -48634,7 +48634,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>People born in the state and counted living in another state at the 2011 census, as a percentage, from Census table D-01 (place of birth). The curated file does not record which population the percentage is of.</t>
+          <t>People born in the state and counted in another Indian state at the 2011 census, as a percentage of the state's own population counted in 2011, from Census table D-01 (place of birth). For Bihar that is 79,49,853 over 10,40,99,452, or 7.64.</t>
         </is>
       </c>
     </row>
@@ -48651,7 +48651,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>People counted living in the state at the 2011 census who were born in another state, as a percentage, from Census table D-01 (place of birth). The curated file does not record which population the percentage is of.</t>
+          <t>People counted in the state at the 2011 census who were born in another Indian state, as a percentage of the state's own population counted in 2011, from Census table D-01 (place of birth). People born outside India are not counted. For Bihar that is 10,66,526 over 10,40,99,452, or 1.02.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Writing pass: colon hinges, bold-first list, filler words, front page boxes
Rewrites the front page's constituency box, 'Who this is for' (plain
sentences in place of bold-first bullets) and the 'How we know' headings,
and fixes colon-hinged sentences in meta descriptions and method notes,
semicolon strings in source notes, and filler words (simply, really, very
different, Key insight, At a glance). Changed strings are retranslated, or
carry their translation where only punctuation changed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FWx24PCx3Jw4SUDQC6oU7o
</commit_message>
<xml_diff>
--- a/downloads/india-all-states.xlsx
+++ b/downloads/india-all-states.xlsx
@@ -60787,7 +60787,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>The Chief Electoral Officer's district and constituency tables of the draft, as published by DeshGujarat on 20 December 2025: 5,08,43,436 before; 18,07,278 death, 9,69,662 untraceable or absent, 40,25,553 permanently shifted, 3,81,470 already enrolled and 1,89,364 other. Shifted, absent or other is absent plus shifted plus other.</t>
+          <t>The Chief Electoral Officer's district and constituency tables of the draft, as published by DeshGujarat on 20 December 2025: 5,08,43,436 before. 18,07,278 death, 9,69,662 untraceable or absent, 40,25,553 permanently shifted, 3,81,470 already enrolled and 1,89,364 other. Shifted, absent or other is absent plus shifted plus other.</t>
         </is>
       </c>
       <c r="Y5" t="n">
@@ -61228,7 +61228,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>The total is the roll before the revision (press note of 16 December 2025) less the draft roll (fact sheet of 21 February 2026), for 199 seats; Anta, which held a by-election, was revised later. The reasons were published only in lakh and sum to 41.79 lakh.</t>
+          <t>The total is the roll before the revision (press note of 16 December 2025) less the draft roll (fact sheet of 21 February 2026), for 199 seats. Anta, which held a by-election, was revised later. The reasons were published only in lakh and sum to 41.79 lakh.</t>
         </is>
       </c>
       <c r="Y8" t="n">
@@ -63196,7 +63196,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>CEO Uttarakhand press note 2026/36 of 14.07.2026: 79,60,762 on 08.06.2026, 71,33,785 on the draft; absent or shifted 6,33,573, deceased 1,24,173, enrolled at more than one place 61,454, others 7,777. Shifted, absent or other is absent or shifted plus others.</t>
+          <t>CEO Uttarakhand press note 2026/36 of 14.07.2026: 79,60,762 on 08.06.2026, 71,33,785 on the draft. Absent or shifted 6,33,573, deceased 1,24,173, enrolled at more than one place 61,454, others 7,777. Shifted, absent or other is absent or shifted plus others.</t>
         </is>
       </c>
       <c r="Y24" t="n">
@@ -63790,7 +63790,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>Only shares of the electorate were reported (absent 22.5%, shifted 4.6%, dead 1.7%, duplicate 0.6%); not converted to counts.</t>
+          <t>Only shares of the electorate were reported (absent 22.5%, shifted 4.6%, dead 1.7%, duplicate 0.6%). Not converted to counts.</t>
         </is>
       </c>
       <c r="AA29" t="n">
@@ -64057,7 +64057,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>CEO Mizoram press note of 4 July 2026: 21,295 dead, 8,333 untraceable, 13,978 shifted, 2,248 already enrolled and 309 others, 46,163 in all; the final press note of 7 September gives 46,162 not received, which is kept as the total.</t>
+          <t>CEO Mizoram press note of 4 July 2026: 21,295 dead, 8,333 untraceable, 13,978 shifted, 2,248 already enrolled and 309 others, 46,163 in all. The final press note of 7 September gives 46,162 not received, which is kept as the total.</t>
         </is>
       </c>
       <c r="AA31" t="n">
@@ -64257,7 +64257,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>Draft roll not yet published; rescheduled to 12 December 2026.</t>
+          <t>Draft roll not yet published. Rescheduled to 12 December 2026.</t>
         </is>
       </c>
       <c r="AE33" t="n">
@@ -72623,7 +72623,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Removals by sex from a press analysis that cites no primary source; the draft roll by sex is the Chief Electoral Officer's.</t>
+          <t>Removals by sex from a press analysis that cites no primary source. The draft roll by sex is the Chief Electoral Officer's.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -72823,7 +72823,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Frozen roll and draft roll by sex (general electors); removals add to the total exactly.</t>
+          <t>Frozen roll and draft roll by sex (general electors). Removals add to the total exactly.</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -72903,7 +72903,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Before and draft rolls by sex, from the Chief Electoral Officer; removals add to the total exactly.</t>
+          <t>Before and draft rolls by sex, from the Chief Electoral Officer. Removals add to the total exactly.</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -72943,7 +72943,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Roll before (15 July 2026) and draft by sex from the official statement reported by PTI; removals by sex are the difference.</t>
+          <t>Roll before (15 July 2026) and draft by sex from the official statement reported by PTI. Removals by sex are the difference.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">

</xml_diff>

<commit_message>
Writing pass across the site, and a named grievance contact (#123)
Rewrites the front page's constituency box, the 'Who this is for' list
(plain sentences in place of bold-first bullets) and the 'How we know'
headings. Fixes colon-hinged sentences in page descriptions and method
notes, semicolon strings in source notes, and filler words. Changed
strings are retranslated or carry their translation where only
punctuation changed.

The terms page now names the editor at PinPoint Ventures as the
grievance contact.

All 49 data checks, the build check, the i18n check (2,704 strings) and
contrast pass.

🤖 Generated with [Claude Code](https://claude.com/claude-code)

https://claude.ai/code/session_01FWx24PCx3Jw4SUDQC6oU7o

---
_Generated by [Claude
Code](https://claude.ai/code/session_01FWx24PCx3Jw4SUDQC6oU7o)_

---------

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/india-all-states.xlsx
+++ b/downloads/india-all-states.xlsx
@@ -60787,7 +60787,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>The Chief Electoral Officer's district and constituency tables of the draft, as published by DeshGujarat on 20 December 2025: 5,08,43,436 before; 18,07,278 death, 9,69,662 untraceable or absent, 40,25,553 permanently shifted, 3,81,470 already enrolled and 1,89,364 other. Shifted, absent or other is absent plus shifted plus other.</t>
+          <t>The Chief Electoral Officer's district and constituency tables of the draft, as published by DeshGujarat on 20 December 2025: 5,08,43,436 before. 18,07,278 death, 9,69,662 untraceable or absent, 40,25,553 permanently shifted, 3,81,470 already enrolled and 1,89,364 other. Shifted, absent or other is absent plus shifted plus other.</t>
         </is>
       </c>
       <c r="Y5" t="n">
@@ -61228,7 +61228,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>The total is the roll before the revision (press note of 16 December 2025) less the draft roll (fact sheet of 21 February 2026), for 199 seats; Anta, which held a by-election, was revised later. The reasons were published only in lakh and sum to 41.79 lakh.</t>
+          <t>The total is the roll before the revision (press note of 16 December 2025) less the draft roll (fact sheet of 21 February 2026), for 199 seats. Anta, which held a by-election, was revised later. The reasons were published only in lakh and sum to 41.79 lakh.</t>
         </is>
       </c>
       <c r="Y8" t="n">
@@ -63196,7 +63196,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>CEO Uttarakhand press note 2026/36 of 14.07.2026: 79,60,762 on 08.06.2026, 71,33,785 on the draft; absent or shifted 6,33,573, deceased 1,24,173, enrolled at more than one place 61,454, others 7,777. Shifted, absent or other is absent or shifted plus others.</t>
+          <t>CEO Uttarakhand press note 2026/36 of 14.07.2026: 79,60,762 on 08.06.2026, 71,33,785 on the draft. Absent or shifted 6,33,573, deceased 1,24,173, enrolled at more than one place 61,454, others 7,777. Shifted, absent or other is absent or shifted plus others.</t>
         </is>
       </c>
       <c r="Y24" t="n">
@@ -63790,7 +63790,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>Only shares of the electorate were reported (absent 22.5%, shifted 4.6%, dead 1.7%, duplicate 0.6%); not converted to counts.</t>
+          <t>Only shares of the electorate were reported (absent 22.5%, shifted 4.6%, dead 1.7%, duplicate 0.6%). Not converted to counts.</t>
         </is>
       </c>
       <c r="AA29" t="n">
@@ -64057,7 +64057,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>CEO Mizoram press note of 4 July 2026: 21,295 dead, 8,333 untraceable, 13,978 shifted, 2,248 already enrolled and 309 others, 46,163 in all; the final press note of 7 September gives 46,162 not received, which is kept as the total.</t>
+          <t>CEO Mizoram press note of 4 July 2026: 21,295 dead, 8,333 untraceable, 13,978 shifted, 2,248 already enrolled and 309 others, 46,163 in all. The final press note of 7 September gives 46,162 not received, which is kept as the total.</t>
         </is>
       </c>
       <c r="AA31" t="n">
@@ -64257,7 +64257,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>Draft roll not yet published; rescheduled to 12 December 2026.</t>
+          <t>Draft roll not yet published. Rescheduled to 12 December 2026.</t>
         </is>
       </c>
       <c r="AE33" t="n">
@@ -72623,7 +72623,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Removals by sex from a press analysis that cites no primary source; the draft roll by sex is the Chief Electoral Officer's.</t>
+          <t>Removals by sex from a press analysis that cites no primary source. The draft roll by sex is the Chief Electoral Officer's.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -72823,7 +72823,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Frozen roll and draft roll by sex (general electors); removals add to the total exactly.</t>
+          <t>Frozen roll and draft roll by sex (general electors). Removals add to the total exactly.</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -72903,7 +72903,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Before and draft rolls by sex, from the Chief Electoral Officer; removals add to the total exactly.</t>
+          <t>Before and draft rolls by sex, from the Chief Electoral Officer. Removals add to the total exactly.</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -72943,7 +72943,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Roll before (15 July 2026) and draft by sex from the official statement reported by PTI; removals by sex are the difference.</t>
+          <t>Roll before (15 July 2026) and draft by sex from the official statement reported by PTI. Removals by sex are the difference.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">

</xml_diff>

<commit_message>
RTI replies page: eleven applications about the SIR, each checked against its source
Lists the applications under the Right to Information Act whose reply,
refusal or appeal was published or reported, with what was asked, what
came back and the days taken. Says plainly that no authority publishes a
count. Pinned on the front page, in the All India menu, search and
downloads.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FWx24PCx3Jw4SUDQC6oU7o
</commit_message>
<xml_diff>
--- a/downloads/india-all-states.xlsx
+++ b/downloads/india-all-states.xlsx
@@ -22,8 +22,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Women, state by state and distr" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rural, mixed and urban district" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protests and disputes" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Every constituency in four stat" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTI replies" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Every constituency in four stat" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1000,33 +1001,68 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
+          <t>RTI replies</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Published table</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>application</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Every application under the Right to Information Act about the revision whose reply was published or reported, with what was asked and what came back</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>A list of the applications that were reported. No authority publishes how many were filed. Each answer is what the outlet reported.</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>data/india/rti.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
           <t>Every constituency in four stat</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Published table</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>constituency</t>
         </is>
       </c>
-      <c r="D20" s="3" t="n">
+      <c r="D21" s="3" t="n">
         <v>738</v>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>Every constituency of Tamil Nadu, Kerala, West Bengal and Uttarakhand in one table</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>Each state measures a different thing, named in the state's rows. Nothing is added across states. Only Uttarakhand has gross additions and deletions.</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>data/india/ac_change.csv</t>
         </is>
@@ -28008,6 +28044,744 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="29" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="48" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>authority</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>applicant</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>filed</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>replied</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>asked</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>outcome</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>answer</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>rti_section</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>All India</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Election Commission of India</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>a transparency activist, co-convenor of the National Campaign for People's Right to Information</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2025-07-28</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2025-08-27</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>A copy of any independent appraisal or study on which the Commission decided to begin the SIR across the country in 2025, and the files, notings and records on that decision, with time to inspect them.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>no record held</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>The Times of India reported that the CPIO pointed to the guidelines of 24 June 2025 and said no further information was available, and The News Minute reported that on first appeal the Commission's Principal Secretary wrote that the Commission had not taken any decision on a nationwide SIR in 2025.</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>The News Minute</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>https://www.thenewsminute.com/news/who-decided-on-nationwide-sir-ecs-rti-response-raises-questions</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>All India</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Election Commission of India</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>My Vote, My Right (a coalition of civil society groups)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>The definition of 'logical discrepancy' in any official document and the number of notices issued to electors in the 10 States and UTs where the SIR was complete.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>no record held</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>The News Minute reported that the Commission said the information was not available with it and might be with the CEOs of the States and UTs.</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>The News Minute</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>https://www.thenewsminute.com/karnataka/eci-has-no-record-of-what-constitutes-logical-discrepancy-in-sir-rti-reply-shows</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Bihar</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Election Commission of India</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>a transparency activist, co-convenor of the National Campaign for People's Right to Information</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2025-07-28</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>The order or notification for the 2003 intensive revision of Bihar's rolls and the guidelines for that revision, including the forms and documents required.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>not supplied</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Deccan Herald and The Times of India reported that the CPIO sent only the link to the 2025 SIR guidelines of 24 June 2025 and gave nothing on the 2003 revision.</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Deccan Herald</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2025-08-28</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>https://www.deccanherald.com/india/election-commission-refuses-to-provide-2003-bihar-sir-order-on-rti-query-3701142</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>All India</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Election Commission of India</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>The Reporters' Collective</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>All files, notings, correspondence, minutes, presentations and drafts on the SIR ordered on 24 June 2025, and a list of the files recording it.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>not supplied</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>The Reporters' Collective reported that the Commission replied with a link to a page of 'comprehensive instructions' dated 14 July 2025 that the outlet could not open, and did not name any file on the decision.</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>The Reporters' Collective</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2025-08-29</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>https://www.reporters-collective.in/blog/a-dead-weblink-eci-refuses-to-share-its-records-under-rti-law</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>West Bengal</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Election Commission of India</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>a Trinamool Congress leader</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>95</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Technical documents on the 'logical discrepancy' module in ERONET used for the West Bengal SIR, its logic and parameters, procurement and testing records, file notings, instructions to EROs, and the number of electors flagged under each sub-category.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>refused</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Deccan Herald (PTI) reported that the Commission held the software questions exempt under Section 8(1)(d), said no module or separate procurement had been made for the West Bengal SIR, and directed the question on flagged electors to the EROs.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>8(1)(d)</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Deccan Herald (PTI)</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>https://www.deccanherald.com/india/west-bengal/tmcs-saket-gokhale-says-ec-withholding-details-of-sir-software-cites-rti-response-4157888</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>All India</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ministry of Law and Justice, transferred to the Election Commission of India</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>The Reporters' Collective</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2025-08-20</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Whether the Commission sought the Law Ministry's legal opinion on the SIR and, if so, the full paper trail of files, correspondence, memos, notes and presentations.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>The Reporters' Collective reported that the Ministry said it keeps no record of such advice and transferred the request to the Commission, which replied on 20 August 2025 that it had no information.</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>The Reporters' Collective</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2025-08-29</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>https://www.reporters-collective.in/blog/a-dead-weblink-eci-refuses-to-share-its-records-under-rti-law</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Bihar</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CEO Bihar, transferred to the 38 DEOs</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>a transparency activist</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>How many times EROs sent speed post notices to absent or shifted electors during the SIR, how many replies they received and how many notices came back undelivered.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>The Reporters' Collective reported that the CEO sent the application to all 38 district election offices and that after eleven months only the Dulhin Bazar subdivision of Patna and the Hajipur district office had replied, the first saying it sent no speed post notices and the second saying electors were marked from the BLOs' door to door survey.</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>The Reporters' Collective</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>https://www.reporters-collective.in/blog/follow-regulations-during-sir-not-in-bihar</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>All India</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Election Commission of India</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>an independent writer</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2025-11-29</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>110</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>File notings on the decision to begin the second phase of the SIR and the minutes of all meetings held on it.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>partly supplied</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>The Wire reported that after a first appeal the Commission supplied two pages of file notings showing the proposal initiated by an Under Secretary on 27 October 2025 and approved the same day, and supplied no minutes of meetings.</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>The Wire</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>https://thewire.in/government/if-voter-rolls-were-properly-maintained-would-sir-be-needed-rti-records-tell-the-story</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>West Bengal</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CEO West Bengal</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>a Congress Member of Parliament from West Bengal</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Figures on appeals before the SIR appellate tribunals in West Bengal, received, decided, allowed and rejected, district by district.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>supplied</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>The Wire reported a 28 page reply, Memo No. 8551/Home (Elec), showing that as of 7 August 2026 the tribunals had received 38,10,620 appeals and decided 82,782, of which 75,443 ended in inclusion and 7,339 in exclusion, with a footnote that the total mixes appeals against inclusion and against exclusion.</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>The Wire</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>https://thewire.in/rights/rti-reveals-bengal-tribunal-decided-on-just-2-17-sir-appeals-over-37-lakh-still-in-limbo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>West Bengal</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Election Commission of India</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>a petitioner in the Calcutta High Court</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>The circular or notification under which the SIR was carried out in West Bengal and any record the Commission holds on foreign nationals on the roll.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>appeal</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>ETV Bharat reported that the CPIO gave no information, that the first appellate authority directed disclosure within seven days and warned on 9 February 2026, and that on 18 March 2026 the Calcutta High Court directed the CPIO to supply the information within seven days.</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>ETV Bharat Bangla</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>https://www.etvbharat.com/bn/state/calcutta-high-court-directs-election-commission-of-india-to-answer-rti-over-sir-circular-in-west-bengal-west-bengal-news-wbs26031805380</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>All India</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Election Commission of India, CEO Delhi, CEO West Bengal</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Internet Freedom Foundation</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>The criteria for flagging 'logical discrepancies' and their version history, contracts for ERONET 2.0, ECINET and roll digitisation, Election Commissioners' recorded objections and minutes, data retention and sharing, and State-wise counts of electors excluded, noticed, deleted and restored on appeal.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Internet Freedom Foundation said it had filed the applications and would publish the responses and appeal any refusal.</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Internet Freedom Foundation</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>https://internetfreedom.in/iff-filed-rti-applications-seeking-what-the-election-commission-has-not-disclosed-about-the-sir/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M739"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -56634,13 +57408,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C197"/>
+  <dimension ref="A1:C211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -59779,7 +60553,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -59789,209 +60563,447 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>The state, one of the four that published their rolls by constituency (Tamil Nadu, Kerala, West Bengal and Uttarakhand).</t>
+          <t>The state the application concerns, or All India for one about the revision as a whole.</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>ac</t>
+          <t>authority</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>The assembly constituency number.</t>
+          <t>The public authority the application went to, such as the Election Commission or a state's Chief Electoral Officer.</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>constituency</t>
+          <t>applicant</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>The assembly constituency's name.</t>
+          <t>The organisation that filed it, or the applicant's role. No private person is named.</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>filed</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>The district the constituency lies in.</t>
+          <t>The date the application was filed, where it was reported.</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>earlier_roll</t>
+          <t>replied</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>The earliest roll in the row, which is the roll of 27 October 2025 worked out as the draft plus the names left off for Tamil Nadu, the January 2025 final roll for Kerala, the 2024 Lok Sabha roll for West Bengal and blank for Uttarakhand.</t>
+          <t>The date of the reply, where it was reported.</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>left_off_draft</t>
+          <t>days</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Names left off the draft, as a count, given by constituency only in Tamil Nadu.</t>
+          <t>Days from the application to the reply, where both dates were reported. The Act allows 30.</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>asked</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Electors on the draft roll (19 December 2025 in Tamil Nadu, 23 December 2025 in Kerala, 16 December 2025 in West Bengal, July 2026 in Uttarakhand).</t>
+          <t>What the application asked for.</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>added_after_draft</t>
+          <t>outcome</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Claims admitted after the draft, as a count, Uttarakhand only, from the Chief Electoral Officer's PN 63/2026.</t>
+          <t>What became of it: no record held, refused, transferred, partly supplied, supplied, appeal, no reply in time or pending.</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>removed_after_draft</t>
+          <t>answer</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Objections admitted after the draft, as a count, Uttarakhand only, from PN 63/2026.</t>
+          <t>What the authority said or did, as reported.</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>later_roll</t>
+          <t>rti_section</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>The latest roll in the row, the final roll of 23 February 2026 in Tamil Nadu, 21 February 2026 in Kerala and 3 October 2026 in Uttarakhand, and the roll at the 2026 nominations in West Bengal.</t>
+          <t>The section of the Act cited for a refusal, if any.</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>change_draft_to_later</t>
+          <t>kind</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>later_roll less draft, a net change that counts new voters added after the draft as well as names put back.</t>
+          <t>primary if the reply itself was read, press if the item rests on a report.</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>change_earlier_to_later</t>
+          <t>source</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>later_roll less earlier_roll, as a count, which is negative where the roll fell.</t>
+          <t>The outlet that published the reply or reported it.</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
+          <t>RTI replies</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>The date of that publication.</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>RTI replies</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>The address of the source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
           <t>Every constituency in four stat</t>
         </is>
       </c>
-      <c r="B197" t="inlineStr">
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>The state, one of the four that published their rolls by constituency (Tamil Nadu, Kerala, West Bengal and Uttarakhand).</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>ac</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>The assembly constituency number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>constituency</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>The assembly constituency's name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>The district the constituency lies in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>earlier_roll</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>The earliest roll in the row, which is the roll of 27 October 2025 worked out as the draft plus the names left off for Tamil Nadu, the January 2025 final roll for Kerala, the 2024 Lok Sabha roll for West Bengal and blank for Uttarakhand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>left_off_draft</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Names left off the draft, as a count, given by constituency only in Tamil Nadu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Electors on the draft roll (19 December 2025 in Tamil Nadu, 23 December 2025 in Kerala, 16 December 2025 in West Bengal, July 2026 in Uttarakhand).</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>added_after_draft</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Claims admitted after the draft, as a count, Uttarakhand only, from the Chief Electoral Officer's PN 63/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>removed_after_draft</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Objections admitted after the draft, as a count, Uttarakhand only, from PN 63/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>later_roll</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>The latest roll in the row, the final roll of 23 February 2026 in Tamil Nadu, 21 February 2026 in Kerala and 3 October 2026 in Uttarakhand, and the roll at the 2026 nominations in West Bengal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>change_draft_to_later</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>later_roll less draft, a net change that counts new voters added after the draft as well as names put back.</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>change_earlier_to_later</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>later_roll less earlier_roll, as a count, which is negative where the roll fell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
         <is>
           <t>change_earlier_to_later_per_100</t>
         </is>
       </c>
-      <c r="C197" t="inlineStr">
+      <c r="C211" t="inlineStr">
         <is>
           <t>change_earlier_to_later per 100 electors on earlier_roll.</t>
         </is>

</xml_diff>

<commit_message>
RTI replies page (#130)
New page india/rti/ listing eleven applications under the Right to
Information Act about the SIR whose reply, refusal or appeal was
published or reported. Each was read by one researcher and checked
against its source by a second (6 confirmed, 5 corrected). The page says
no authority publishes a count of such applications. Pinned on the front
page, added to the All India menu and tab row, the sitewide search, the
downloads (CSV) and the FAQ. Builder scripts/build_rti.py, checked by
check_data.py.

🤖 Generated with [Claude Code](https://claude.com/claude-code)

https://claude.ai/code/session_01FWx24PCx3Jw4SUDQC6oU7o

---
_Generated by [Claude
Code](https://claude.ai/code/session_01FWx24PCx3Jw4SUDQC6oU7o)_

---------

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/india-all-states.xlsx
+++ b/downloads/india-all-states.xlsx
@@ -22,8 +22,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Women, state by state and distr" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rural, mixed and urban district" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protests and disputes" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Every constituency in four stat" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTI replies" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Every constituency in four stat" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1000,33 +1001,68 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
+          <t>RTI replies</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Published table</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>application</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Every application under the Right to Information Act about the revision whose reply was published or reported, with what was asked and what came back</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>A list of the applications that were reported. No authority publishes how many were filed. Each answer is what the outlet reported.</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>data/india/rti.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
           <t>Every constituency in four stat</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Published table</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>constituency</t>
         </is>
       </c>
-      <c r="D20" s="3" t="n">
+      <c r="D21" s="3" t="n">
         <v>738</v>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>Every constituency of Tamil Nadu, Kerala, West Bengal and Uttarakhand in one table</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>Each state measures a different thing, named in the state's rows. Nothing is added across states. Only Uttarakhand has gross additions and deletions.</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>data/india/ac_change.csv</t>
         </is>
@@ -28008,6 +28044,744 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="29" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="48" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>authority</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>applicant</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>filed</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>replied</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>asked</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>outcome</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>answer</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>rti_section</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>All India</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Election Commission of India</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>a transparency activist, co-convenor of the National Campaign for People's Right to Information</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2025-07-28</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2025-08-27</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>A copy of any independent appraisal or study on which the Commission decided to begin the SIR across the country in 2025, and the files, notings and records on that decision, with time to inspect them.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>no record held</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>The Times of India reported that the CPIO pointed to the guidelines of 24 June 2025 and said no further information was available, and The News Minute reported that on first appeal the Commission's Principal Secretary wrote that the Commission had not taken any decision on a nationwide SIR in 2025.</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>The News Minute</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>https://www.thenewsminute.com/news/who-decided-on-nationwide-sir-ecs-rti-response-raises-questions</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>All India</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Election Commission of India</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>My Vote, My Right (a coalition of civil society groups)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>The definition of 'logical discrepancy' in any official document and the number of notices issued to electors in the 10 States and UTs where the SIR was complete.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>no record held</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>The News Minute reported that the Commission said the information was not available with it and might be with the CEOs of the States and UTs.</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>The News Minute</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>https://www.thenewsminute.com/karnataka/eci-has-no-record-of-what-constitutes-logical-discrepancy-in-sir-rti-reply-shows</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Bihar</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Election Commission of India</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>a transparency activist, co-convenor of the National Campaign for People's Right to Information</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2025-07-28</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>The order or notification for the 2003 intensive revision of Bihar's rolls and the guidelines for that revision, including the forms and documents required.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>not supplied</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Deccan Herald and The Times of India reported that the CPIO sent only the link to the 2025 SIR guidelines of 24 June 2025 and gave nothing on the 2003 revision.</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Deccan Herald</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2025-08-28</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>https://www.deccanherald.com/india/election-commission-refuses-to-provide-2003-bihar-sir-order-on-rti-query-3701142</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>All India</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Election Commission of India</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>The Reporters' Collective</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>All files, notings, correspondence, minutes, presentations and drafts on the SIR ordered on 24 June 2025, and a list of the files recording it.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>not supplied</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>The Reporters' Collective reported that the Commission replied with a link to a page of 'comprehensive instructions' dated 14 July 2025 that the outlet could not open, and did not name any file on the decision.</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>The Reporters' Collective</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2025-08-29</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>https://www.reporters-collective.in/blog/a-dead-weblink-eci-refuses-to-share-its-records-under-rti-law</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>West Bengal</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Election Commission of India</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>a Trinamool Congress leader</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>95</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Technical documents on the 'logical discrepancy' module in ERONET used for the West Bengal SIR, its logic and parameters, procurement and testing records, file notings, instructions to EROs, and the number of electors flagged under each sub-category.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>refused</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Deccan Herald (PTI) reported that the Commission held the software questions exempt under Section 8(1)(d), said no module or separate procurement had been made for the West Bengal SIR, and directed the question on flagged electors to the EROs.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>8(1)(d)</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Deccan Herald (PTI)</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>https://www.deccanherald.com/india/west-bengal/tmcs-saket-gokhale-says-ec-withholding-details-of-sir-software-cites-rti-response-4157888</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>All India</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ministry of Law and Justice, transferred to the Election Commission of India</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>The Reporters' Collective</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2025-08-20</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Whether the Commission sought the Law Ministry's legal opinion on the SIR and, if so, the full paper trail of files, correspondence, memos, notes and presentations.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>The Reporters' Collective reported that the Ministry said it keeps no record of such advice and transferred the request to the Commission, which replied on 20 August 2025 that it had no information.</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>The Reporters' Collective</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2025-08-29</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>https://www.reporters-collective.in/blog/a-dead-weblink-eci-refuses-to-share-its-records-under-rti-law</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Bihar</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CEO Bihar, transferred to the 38 DEOs</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>a transparency activist</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>How many times EROs sent speed post notices to absent or shifted electors during the SIR, how many replies they received and how many notices came back undelivered.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>The Reporters' Collective reported that the CEO sent the application to all 38 district election offices and that after eleven months only the Dulhin Bazar subdivision of Patna and the Hajipur district office had replied, the first saying it sent no speed post notices and the second saying electors were marked from the BLOs' door to door survey.</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>The Reporters' Collective</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>https://www.reporters-collective.in/blog/follow-regulations-during-sir-not-in-bihar</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>All India</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Election Commission of India</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>an independent writer</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2025-11-29</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>110</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>File notings on the decision to begin the second phase of the SIR and the minutes of all meetings held on it.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>partly supplied</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>The Wire reported that after a first appeal the Commission supplied two pages of file notings showing the proposal initiated by an Under Secretary on 27 October 2025 and approved the same day, and supplied no minutes of meetings.</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>The Wire</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>https://thewire.in/government/if-voter-rolls-were-properly-maintained-would-sir-be-needed-rti-records-tell-the-story</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>West Bengal</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CEO West Bengal</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>a Congress Member of Parliament from West Bengal</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Figures on appeals before the SIR appellate tribunals in West Bengal, received, decided, allowed and rejected, district by district.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>supplied</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>The Wire reported a 28 page reply, Memo No. 8551/Home (Elec), showing that as of 7 August 2026 the tribunals had received 38,10,620 appeals and decided 82,782, of which 75,443 ended in inclusion and 7,339 in exclusion, with a footnote that the total mixes appeals against inclusion and against exclusion.</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>The Wire</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>https://thewire.in/rights/rti-reveals-bengal-tribunal-decided-on-just-2-17-sir-appeals-over-37-lakh-still-in-limbo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>West Bengal</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Election Commission of India</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>a petitioner in the Calcutta High Court</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>The circular or notification under which the SIR was carried out in West Bengal and any record the Commission holds on foreign nationals on the roll.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>appeal</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>ETV Bharat reported that the CPIO gave no information, that the first appellate authority directed disclosure within seven days and warned on 9 February 2026, and that on 18 March 2026 the Calcutta High Court directed the CPIO to supply the information within seven days.</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>ETV Bharat Bangla</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>https://www.etvbharat.com/bn/state/calcutta-high-court-directs-election-commission-of-india-to-answer-rti-over-sir-circular-in-west-bengal-west-bengal-news-wbs26031805380</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>All India</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Election Commission of India, CEO Delhi, CEO West Bengal</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Internet Freedom Foundation</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>The criteria for flagging 'logical discrepancies' and their version history, contracts for ERONET 2.0, ECINET and roll digitisation, Election Commissioners' recorded objections and minutes, data retention and sharing, and State-wise counts of electors excluded, noticed, deleted and restored on appeal.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Internet Freedom Foundation said it had filed the applications and would publish the responses and appeal any refusal.</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Internet Freedom Foundation</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>https://internetfreedom.in/iff-filed-rti-applications-seeking-what-the-election-commission-has-not-disclosed-about-the-sir/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M739"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -56634,13 +57408,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C197"/>
+  <dimension ref="A1:C211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -59779,7 +60553,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -59789,209 +60563,447 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>The state, one of the four that published their rolls by constituency (Tamil Nadu, Kerala, West Bengal and Uttarakhand).</t>
+          <t>The state the application concerns, or All India for one about the revision as a whole.</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>ac</t>
+          <t>authority</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>The assembly constituency number.</t>
+          <t>The public authority the application went to, such as the Election Commission or a state's Chief Electoral Officer.</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>constituency</t>
+          <t>applicant</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>The assembly constituency's name.</t>
+          <t>The organisation that filed it, or the applicant's role. No private person is named.</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>filed</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>The district the constituency lies in.</t>
+          <t>The date the application was filed, where it was reported.</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>earlier_roll</t>
+          <t>replied</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>The earliest roll in the row, which is the roll of 27 October 2025 worked out as the draft plus the names left off for Tamil Nadu, the January 2025 final roll for Kerala, the 2024 Lok Sabha roll for West Bengal and blank for Uttarakhand.</t>
+          <t>The date of the reply, where it was reported.</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>left_off_draft</t>
+          <t>days</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Names left off the draft, as a count, given by constituency only in Tamil Nadu.</t>
+          <t>Days from the application to the reply, where both dates were reported. The Act allows 30.</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>asked</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Electors on the draft roll (19 December 2025 in Tamil Nadu, 23 December 2025 in Kerala, 16 December 2025 in West Bengal, July 2026 in Uttarakhand).</t>
+          <t>What the application asked for.</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>added_after_draft</t>
+          <t>outcome</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Claims admitted after the draft, as a count, Uttarakhand only, from the Chief Electoral Officer's PN 63/2026.</t>
+          <t>What became of it: no record held, refused, transferred, partly supplied, supplied, appeal, no reply in time or pending.</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>removed_after_draft</t>
+          <t>answer</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Objections admitted after the draft, as a count, Uttarakhand only, from PN 63/2026.</t>
+          <t>What the authority said or did, as reported.</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>later_roll</t>
+          <t>rti_section</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>The latest roll in the row, the final roll of 23 February 2026 in Tamil Nadu, 21 February 2026 in Kerala and 3 October 2026 in Uttarakhand, and the roll at the 2026 nominations in West Bengal.</t>
+          <t>The section of the Act cited for a refusal, if any.</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>change_draft_to_later</t>
+          <t>kind</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>later_roll less draft, a net change that counts new voters added after the draft as well as names put back.</t>
+          <t>primary if the reply itself was read, press if the item rests on a report.</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Every constituency in four stat</t>
+          <t>RTI replies</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>change_earlier_to_later</t>
+          <t>source</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>later_roll less earlier_roll, as a count, which is negative where the roll fell.</t>
+          <t>The outlet that published the reply or reported it.</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
+          <t>RTI replies</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>The date of that publication.</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>RTI replies</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>The address of the source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
           <t>Every constituency in four stat</t>
         </is>
       </c>
-      <c r="B197" t="inlineStr">
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>The state, one of the four that published their rolls by constituency (Tamil Nadu, Kerala, West Bengal and Uttarakhand).</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>ac</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>The assembly constituency number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>constituency</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>The assembly constituency's name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>The district the constituency lies in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>earlier_roll</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>The earliest roll in the row, which is the roll of 27 October 2025 worked out as the draft plus the names left off for Tamil Nadu, the January 2025 final roll for Kerala, the 2024 Lok Sabha roll for West Bengal and blank for Uttarakhand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>left_off_draft</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Names left off the draft, as a count, given by constituency only in Tamil Nadu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Electors on the draft roll (19 December 2025 in Tamil Nadu, 23 December 2025 in Kerala, 16 December 2025 in West Bengal, July 2026 in Uttarakhand).</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>added_after_draft</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Claims admitted after the draft, as a count, Uttarakhand only, from the Chief Electoral Officer's PN 63/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>removed_after_draft</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Objections admitted after the draft, as a count, Uttarakhand only, from PN 63/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>later_roll</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>The latest roll in the row, the final roll of 23 February 2026 in Tamil Nadu, 21 February 2026 in Kerala and 3 October 2026 in Uttarakhand, and the roll at the 2026 nominations in West Bengal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>change_draft_to_later</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>later_roll less draft, a net change that counts new voters added after the draft as well as names put back.</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>change_earlier_to_later</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>later_roll less earlier_roll, as a count, which is negative where the roll fell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Every constituency in four stat</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
         <is>
           <t>change_earlier_to_later_per_100</t>
         </is>
       </c>
-      <c r="C197" t="inlineStr">
+      <c r="C211" t="inlineStr">
         <is>
           <t>change_earlier_to_later per 100 electors on earlier_roll.</t>
         </is>

</xml_diff>

<commit_message>
Karnataka: roll of 9 October 2026; Jharkhand final roll moved to 30 November; Telangana's exact roll before
Karnataka's pages, report and deck move from the roll of 25 September to the
CEO's press note of 9 October (45,161,393 electors, by district and sex),
with its notices and forms tables added to raw and the downloads. The state
row is matched to the press; the district rows add exactly to it.
Jharkhand's final roll date follows the CEO as quoted by Town Post (30
November). Telangana's roll before the revision is 3,38,26,448 (Telangana
Today, from the CEO), replacing the rounded 3.38 crore. The figures-as-of
line now reads moved dates, and the place name above each heading uses the
normal type in non-Latin scripts.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FWx24PCx3Jw4SUDQC6oU7o
</commit_message>
<xml_diff>
--- a/downloads/india-all-states.xlsx
+++ b/downloads/india-all-states.xlsx
@@ -63327,13 +63327,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>33800000</v>
+        <v>33826448</v>
       </c>
       <c r="E17" t="n">
         <v>7339235</v>
       </c>
       <c r="F17" t="n">
-        <v>21.71</v>
+        <v>21.7</v>
       </c>
       <c r="G17" t="n">
         <v>922229</v>
@@ -63354,7 +63354,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>rounded</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -63369,7 +63369,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>Electors before the revision reported rounded (3.38 crore).</t>
+          <t>Removals and reasons from The Indian Express. The roll before the revision, 3,38,26,448, is from Telangana Today of 9 October 2026, from the Chief Electoral Officer's information, with 2,64,87,213 enumeration forms submitted and 73,39,235 left off (https://telanganatoday.com/telangana-sir-18-12-lakh-voters-face-exclusion-from-final-electoral-list).</t>
         </is>
       </c>
       <c r="Y17" t="n">
@@ -79507,7 +79507,7 @@
         <v>3</v>
       </c>
       <c r="C3" t="n">
-        <v>26460765</v>
+        <v>26487213</v>
       </c>
       <c r="D3" t="n">
         <v>9288180</v>

</xml_diff>

<commit_message>
Fix All India fact-check findings: private names, notices, counts from data
- process.json: private voters, BLOs and the deceased named by role; disputes rebuilt
- Uttarakhand notices: 20.27 lakh served (24.30 lakh was the target)
- Phase III moved-date count and claims-after-draft burden computed from data
- 20 Feb 2026 timeline entry split; 24 Feb entry from the 10 Mar order
- Mihir Rajesh Shah cited by appeal number and SCC only
- women over-represented counted by plain comparison (8 of 11)
- Maharashtra and Delhi rows cite the CEO press notes; Territories limits computed
- West Bengal adjudication outcomes, as reported; as_of derived from the data
- Not split is the sum of shortfalls; one half-up rounding (SIR.d, report)
- method, numbers, progress, front page and report/deck source text corrected

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FWx24PCx3Jw4SUDQC6oU7o
</commit_message>
<xml_diff>
--- a/downloads/india-all-states.xlsx
+++ b/downloads/india-all-states.xlsx
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
@@ -27536,12 +27536,12 @@
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>The Wire reported that Mintu Paswan of Ara, Bhojpur, who had been declared dead in the Bihar draft roll, appeared alive in the Supreme Court on 12 August 2025, produced by petitioner Yogendra Yadav. Paswan told The Wire he had filled the enumeration form and that the BLO came to his house only after he complained.</t>
+          <t>The Wire reported that a voter from Ara, Bhojpur, who had been declared dead in the Bihar draft roll, appeared alive in the Supreme Court on 12 August 2025, produced by petitioner Yogendra Yadav. The voter told The Wire he had filled the enumeration form and that the BLO came to his house only after he complained.</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>Senior advocate Rakesh Dwivedi, for the Commission, called the production of Paswan "drama". The bench of Justices Surya Kant and Joymalya Bagchi said there may have been an "inadvertent error", which could be rectified.</t>
+          <t>Senior advocate Rakesh Dwivedi, for the Commission, called the production of the voter "drama". The bench of Justices Surya Kant and Joymalya Bagchi said there may have been an "inadvertent error", which could be rectified.</t>
         </is>
       </c>
       <c r="L156" t="inlineStr">
@@ -27598,7 +27598,7 @@
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>Parth Gupta, electoral registration officer for Purnia, acknowledged that Jhurana Das should not have been asked for her parents' documents, and said, “Please provide her details and I will look into it.” Scroll also reported that Election Commission spokespersons and Bihar Chief Electoral Officer Vinod Singh Gunjiyal did not respond to requests for comment.</t>
+          <t>Parth Gupta, electoral registration officer for Purnia, acknowledged that one deleted voter should not have been asked for her parents' documents, and said, “Please provide her details and I will look into it.” Scroll also reported that Election Commission spokespersons and Bihar Chief Electoral Officer Vinod Singh Gunjiyal did not respond to requests for comment.</t>
         </is>
       </c>
       <c r="L157" t="inlineStr">
@@ -27806,7 +27806,7 @@
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>The Indian Express reported the deaths of two BLOs. The family of Aneesh George in Kannur, Kerala, alleged he was under pressure to finish by December 4, and police said a note found on Mukesh Jangid in Jaipur said he faced extreme pressure from his supervisor and was told he would be suspended if he did not meet his SIR target. It also reported that revenue employees in Tamil Nadu announced a statewide boycott of SIR work over workload.</t>
+          <t>The Indian Express reported the deaths of two BLOs. The family of a BLO in Kannur, Kerala, alleged he was under pressure to finish by December 4, and police said a note found on a BLO in Jaipur said he faced extreme pressure from his supervisor and was told he would be suspended if he did not meet his SIR target. It also reported that revenue employees in Tamil Nadu announced a statewide boycott of SIR work over workload.</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -27863,7 +27863,7 @@
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>The Indian Express reported that two women assistant BLOs died of heart attacks in Tapi and Vadodara districts, bringing BLO deaths in Gujarat that week to four. The husband of one, Usha Solanki, said she was a heart patient who had asked to be excused from BLO duty, which the Vadodara Collector disputed.</t>
+          <t>The Indian Express reported that two women assistant BLOs died of heart attacks in Tapi and Vadodara districts, bringing BLO deaths in Gujarat that week to four. The husband of one said she was a heart patient who had asked to be excused from BLO duty, which the Vadodara Collector disputed.</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -27972,7 +27972,7 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>The Indian Express reported that Kanchan Kumar Mondal, 75, died of cardiac arrest, according to hospital sources, after falling ill in a queue for an SIR hearing at the Rampurhat-1 block office in Birbhum. His wife and family alleged the SIR process had caused him excessive stress and held the Election Commission responsible. It also reported that Madan Ghosh died of cardiac arrest at an SIR hearing in Howrah the previous day.</t>
+          <t>The Indian Express reported that a 75-year-old man died of cardiac arrest, according to hospital sources, after falling ill in a queue for an SIR hearing at the Rampurhat-1 block office in Birbhum. His wife and family alleged the SIR process had caused him excessive stress and held the Election Commission responsible. It also reported that an elderly man died of cardiac arrest at an SIR hearing in Howrah the previous day.</t>
         </is>
       </c>
       <c r="L164" t="inlineStr">
@@ -28024,7 +28024,7 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>The New Indian Express, citing PTI, reported that police in Purulia registered an FIR on a complaint by the son of Durjan Majhi, 82, who died allegedly by suicide on 29 December hours before he was due at an SIR hearing. An officer was quoted as saying the case included charges of abetment of suicide and criminal conspiracy against Election Commission officials, with no official named. The family alleged he acted out of anxiety over the SIR.</t>
+          <t>The New Indian Express, citing PTI, reported that police in Purulia registered an FIR on a complaint by the son of an 82-year-old man who died allegedly by suicide on 29 December hours before he was due at an SIR hearing. An officer was quoted as saying the case included charges of abetment of suicide and criminal conspiracy against Election Commission officials, with no official named. The family alleged he acted out of anxiety over the SIR.</t>
         </is>
       </c>
       <c r="L165" t="inlineStr">
@@ -63126,17 +63126,17 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>press</t>
+          <t>primary</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>https://indianexpress.com/article/cities/mumbai/maharashtra-draft-electoral-rolls-sir-2-crore-voters-excluded-claims-objections-portal-10857667/</t>
+          <t>https://ceoelection.maharashtra.gov.in/Downloads/PDF/Notification/Press%20Note%20English_31.08.2026%20Draft%20Roll.pdf</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>Electors before (9,78,54,049), the draft (7,71,65,562) and the names left off (2,06,88,487) are the Chief Electoral Officer's press note of 31 August 2026, which gives no numbers by reason. The reasons are as reported in lakh by the press and sum 10,513 more than the total. Includes 2.23 lakh "others".</t>
+          <t>Electors before (9,78,54,049), the draft (7,71,65,562) and the names left off (2,06,88,487) are the Chief Electoral Officer's press note of 31 August 2026, which gives no numbers by reason. The reasons are as The Indian Express reported them in lakh, and sum 10,513 more than the total. Includes 2.23 lakh "others".</t>
         </is>
       </c>
       <c r="Y15" t="n">
@@ -63369,7 +63369,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>Removals and reasons from The Indian Express. The roll before the revision, 3,38,26,448, is from Telangana Today of 9 October 2026, from the Chief Electoral Officer's information, with 2,64,87,213 enumeration forms submitted and 73,39,235 left off (https://telanganatoday.com/telangana-sir-18-12-lakh-voters-face-exclusion-from-final-electoral-list).</t>
+          <t>Removals and reasons from The Indian Express. The roll before the revision, 3,38,26,448, is from Telangana Today of 9 October 2026, from the Chief Electoral Officer's information, with 2,64,87,213 enumeration forms submitted and 73,39,235 left off.</t>
         </is>
       </c>
       <c r="Y17" t="n">
@@ -63464,17 +63464,17 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>press</t>
+          <t>primary</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>https://www.hindustantimes.com/cities/delhi-news/delhi-sir-narrows-gender-gap-as-voter-roll-shrinks-328-101788200888661.html</t>
+          <t>https://ceodelhi.gov.in/PDFFolders/2026/Draft_PublicationSIR31Aug2026.pdf</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>The Chief Electoral Officer's press note of 31 August 2026, quoted to the elector by Hindustan Times and Business Standard. Claims and objections extended to 30 October 2026.</t>
+          <t>The Chief Electoral Officer's press note of 31 August 2026, which Hindustan Times and Business Standard also quoted to the elector. Claims and objections extended to 30 October 2026.</t>
         </is>
       </c>
       <c r="Y18" t="n">
@@ -73875,7 +73875,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Chief Electoral Officer's statement of the roll before and the draft by sex.</t>
+          <t>The roll before by sex as Hindustan Times quoted the Chief Electoral Officer</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -73975,7 +73975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -74824,29 +74824,29 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Using its powers under Article 142, and with the parties' consent, the Court gave the deciding of claims and objections about inclusion to judicial officers of West Bengal, helped by judicial officers from Jharkhand and Odisha, acting "for and on behalf of this Court". This account of the order comes from the Court's orders of 2 and 13 April 2026.</t>
+          <t>Using its powers under Article 142, and with the parties' consent, the Court gave the deciding of claims and objections about inclusion to judicial officers of West Bengal, acting "for and on behalf of this Court". This account of the order comes from the Court's orders of 2 and 13 April 2026.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Supreme Court order of 13.04.2026</t>
+          <t>Supreme Court order of 02.04.2026 | Supreme Court order of 13.04.2026</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://api.sci.gov.in/supremecourt/2025/64235/64235_2025_1_53_70166_Order_13-Apr-2026.pdf</t>
+          <t>https://api.sci.gov.in/supremecourt/2026/19822/19822_2026_1_51_69596_Order_02-Apr-2026.pdf | https://api.sci.gov.in/supremecourt/2025/64235/64235_2025_1_53_70166_Order_13-Apr-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>State election officer</t>
+          <t>Supreme Court</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -74856,34 +74856,34 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>West Bengal's final roll, with 60 lakh held back</t>
+          <t>Judges from Jharkhand and Odisha, and no appeal to officials</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>The final roll was published with 60,06,675 names marked "under adjudication". They were to be added by a supplementary list if the judicial officers approved them.</t>
+          <t>A further order set out the work given to the judicial officers and said their orders could not be appealed before any executive or administrative officer. Judicial officers from Odisha and Jharkhand joined those of West Bengal, and by 10 March there were 200 of them beside more than 500 from West Bengal. This account of the order comes from the Court's order of 10 March 2026.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>CEO West Bengal, press note CEO/PN-05/2026</t>
+          <t>Supreme Court order of 10.03.2026</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://ceowestbengal.wb.gov.in/Downloads/News/Final%20Press%20Note%20CEO-PN-05-2026.pdf</t>
+          <t>https://api.sci.gov.in/supremecourt/2025/64235/64235_2025_1_42_69352_Order_10-Mar-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Supreme Court</t>
+          <t>State election officer</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -74893,29 +74893,29 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Appeals go to tribunals</t>
+          <t>West Bengal's final roll, with 60 lakh held back</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>No executive officer could hear an appeal against an order of the judicial officers. Appeals were to go to tribunals of former Chief Justices and judges, which the Commission would notify in consultation with the Chief Justice of the Calcutta High Court.</t>
+          <t>The final roll was published with 60,06,675 names marked "under adjudication". They were to be added by a supplementary list if the judicial officers approved them.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Supreme Court order of 10.03.2026</t>
+          <t>CEO West Bengal, press note CEO/PN-05/2026</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://api.sci.gov.in/supremecourt/2025/64235/64235_2025_1_42_69352_Order_10-Mar-2026.pdf</t>
+          <t>https://ceowestbengal.wb.gov.in/Downloads/News/Final%20Press%20Note%20CEO-PN-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -74930,140 +74930,140 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Nineteen tribunals</t>
+          <t>Appeals go to tribunals</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Nineteen appellate tribunals were at work. Appeals decided by 21 and 27 April were to take effect through a supplementary roll before polling, and a pending appeal gave no right to vote.</t>
+          <t>No executive officer could hear an appeal against an order of the judicial officers. Appeals were to go to tribunals of former Chief Justices and judges, which the Commission would notify in consultation with the Chief Justice of the Calcutta High Court.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Supreme Court order of 13.04.2026</t>
+          <t>Supreme Court order of 10.03.2026</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://api.sci.gov.in/supremecourt/2025/64235/64235_2025_1_53_70166_Order_13-Apr-2026.pdf</t>
+          <t>https://api.sci.gov.in/supremecourt/2025/64235/64235_2025_1_42_69352_Order_10-Mar-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Election Commission</t>
+          <t>Supreme Court</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Phase III</t>
+          <t>West Bengal</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>The rest of the country</t>
+          <t>Nineteen tribunals</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>The revision was ordered in 16 states and 3 union territories, covering the whole country except Himachal Pradesh, Jammu and Kashmir and Ladakh, whose dates would be announced later. Eight separate schedules were set. After the draft, notices would go to those who could not be linked to the last intensive revision (the no-mapping list) and to those whose link showed a discrepancy. Lists of those sent notices were to be published.</t>
+          <t>Nineteen appellate tribunals were at work. Appeals decided by 21 and 27 April were to take effect through a supplementary roll before polling, and a pending appeal gave no right to vote.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>ECI press note ECI/PN/086/2026 of 14.05.2026 (PIB) | Copy of the ECI order of 14.05.2026 (district site)</t>
+          <t>Supreme Court order of 13.04.2026</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleasePage.aspx?PRID=2260955&amp;reg=3&amp;lang=1 | https://cdn.s3waas.gov.in/s3ffeabd223de0d4eacb9a3e6e53e5448d/uploads/2026/05/17797105172741.pdf</t>
+          <t>https://api.sci.gov.in/supremecourt/2025/64235/64235_2025_1_53_70166_Order_13-Apr-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Supreme Court</t>
+          <t>Election Commission</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Bihar</t>
+          <t>Phase III</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>The Supreme Court upholds the revision</t>
+          <t>The rest of the country</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>The Court disposed of the petitions. It held that the revision has its legal basis in section 21(3) of the Representation of the People Act read with Article 324, that it was proportionate, and that its document list, with Aadhaar added, was not arbitrary. The Commission may enquire into citizenship only for electoral purposes and must refer doubtful cases to the competent authority of the Central Government. People domiciled in Bihar whose names were wrongly deleted as absent, dead, shifted or duplicate may seek judicial review.</t>
+          <t>The revision was ordered in 16 states and 3 union territories, covering the whole country except Himachal Pradesh, Jammu and Kashmir and Ladakh, whose dates would be announced later. Eight separate schedules were set. After the draft, notices would go to those who could not be linked to the last intensive revision (the no-mapping list) and to those whose link showed a discrepancy. Lists of those sent notices were to be published.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Supreme Court, judgment of 27.05.2026, 2026 INSC 564</t>
+          <t>ECI press note ECI/PN/086/2026 of 14.05.2026 (PIB) | Copy of the ECI order of 14.05.2026 (district site)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://api.sci.gov.in/supremecourt/2025/35785/35785_2025_1_1501_71617_Judgement_27-May-2026.pdf</t>
+          <t>https://www.pib.gov.in/PressReleasePage.aspx?PRID=2260955&amp;reg=3&amp;lang=1 | https://cdn.s3waas.gov.in/s3ffeabd223de0d4eacb9a3e6e53e5448d/uploads/2026/05/17797105172741.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>State election officer</t>
+          <t>Supreme Court</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Phase III</t>
+          <t>Bihar</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Mizoram avoids Sundays</t>
+          <t>The Supreme Court upholds the revision</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>At its Chief Electoral Officer's request, Mizoram's draft moved from Sunday 5 July to 4 July 2026, and its final roll from Sunday 6 September to 7 September.</t>
+          <t>The Court disposed of the petitions. It held that the revision has its legal basis in section 21(3) of the Representation of the People Act read with Article 324, that it was proportionate, and that its document list, with Aadhaar added, was not arbitrary. The Commission may enquire into citizenship only for electoral purposes and must refer doubtful cases to the competent authority of the Central Government. People domiciled in Bihar whose names were wrongly deleted as absent, dead, shifted or duplicate may seek judicial review.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>CEO Mizoram press note of 04.07.2026 | CEO Mizoram press releases</t>
+          <t>Supreme Court, judgment of 27.05.2026, 2026 INSC 564</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://ceo.mizoram.gov.in/storage/press-releases/July_2026/01KWPBBZRST6PJEWCKV628GVGK.pdf | https://ceo.mizoram.gov.in/show-all-data/press-release</t>
+          <t>https://api.sci.gov.in/supremecourt/2025/35785/35785_2025_1_1501_71617_Judgement_27-May-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -75078,29 +75078,29 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Karnataka three weeks later</t>
+          <t>Mizoram avoids Sundays</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Karnataka's draft came out on 24 August 2026 instead of 5 August. Enumeration ran to 17 August, claims to 23 September, and the final roll is due on 27 October instead of 7 October.</t>
+          <t>At its Chief Electoral Officer's request, Mizoram's draft moved from Sunday 5 July to 4 July 2026, and its final roll from Sunday 6 September to 7 September.</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>CEO Karnataka press note of 24.08.2026</t>
+          <t>CEO Mizoram press note of 04.07.2026 | CEO Mizoram press releases</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://ceo.karnataka.gov.in/uploads/PRESS%20NOTE%2024th%20Aug.pdf</t>
+          <t>https://ceo.mizoram.gov.in/storage/press-releases/July_2026/01KWPBBZRST6PJEWCKV628GVGK.pdf | https://ceo.mizoram.gov.in/show-all-data/press-release</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -75115,34 +75115,34 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Maharashtra four weeks later</t>
+          <t>Karnataka three weeks later</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Maharashtra's draft came out on 31 August 2026 instead of 5 August. Claims run to 30 September, and the final roll is due on 4 November instead of 7 October.</t>
+          <t>Karnataka's draft came out on 24 August 2026 instead of 5 August. Enumeration ran to 17 August, claims to 23 September, and the final roll is due on 27 October instead of 7 October.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>CEO Maharashtra press note of 31.08.2026</t>
+          <t>CEO Karnataka press note of 24.08.2026</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://ceoelection.maharashtra.gov.in/Downloads/PDF/Notification/Press%20Note%20English_31.08.2026%20Draft%20Roll.pdf</t>
+          <t>https://ceo.karnataka.gov.in/uploads/PRESS%20NOTE%2024th%20Aug.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Election Commission</t>
+          <t>State election officer</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -75152,29 +75152,29 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Documents at the door, and a drive for those left off</t>
+          <t>Maharashtra four weeks later</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>For people sent notices as unmapped or for logical discrepancies, BLOs would collect documents at home and upload them for the registration officer, so these people need not come to the office. A hearing would be held only in exceptional cases, as the registration officer decides, preferably online, and a family member authorised by the elector could attend. The Commission said the declaration attached to Form 6 for the revision had been upheld by the Supreme Court, and that outside the revision the forms in the Registration of Electors Rules, 1960 apply. Claims were extended in Delhi to 30 October and in Maharashtra to 12 October 2026. Where the revision was complete, in 20 states and union territories, anyone left out during it or after, and any young or first-time voter, could ask the registration officer to be added under continuous updation, and the Chief Electoral Officers, district officers and registration officers were to launch a special drive at once to enrol them.</t>
+          <t>Maharashtra's draft came out on 31 August 2026 instead of 5 August. Claims run to 30 September, and the final roll is due on 4 November instead of 7 October.</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>ECI press note ECI/PN/120/2026 of 26.09.2026 | ECI press release of 26.09.2026 (PIB)</t>
+          <t>CEO Maharashtra press note of 31.08.2026</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.eci.gov.in/eci/public/api/document?id=17536 | https://www.pib.gov.in/PressReleasePage.aspx?PRID=2315309&amp;reg=3&amp;lang=1</t>
+          <t>https://ceoelection.maharashtra.gov.in/Downloads/PDF/Notification/Press%20Note%20English_31.08.2026%20Draft%20Roll.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -75189,29 +75189,29 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Andhra Pradesh and Meghalaya extended</t>
+          <t>Documents at the door, and a drive for those left off</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Andhra Pradesh's notices run to 10 October and its final roll is due on 16 October 2026. Meghalaya's final roll moves to 26 October 2026.</t>
+          <t>For people sent notices as unmapped or for logical discrepancies, BLOs would collect documents at home and upload them for the registration officer, so these people need not come to the office. A hearing would be held only in exceptional cases, as the registration officer decides, preferably online, and a family member authorised by the elector could attend. The Commission said the declaration attached to Form 6 for the revision had been upheld by the Supreme Court, and that outside the revision the forms in the Registration of Electors Rules, 1960 apply. Claims were extended in Delhi to 30 October and in Maharashtra to 12 October 2026. Where the revision was complete, in 20 states and union territories, anyone left out during it or after, and any young or first-time voter, could ask the registration officer to be added under continuous updation, and the Chief Electoral Officers, district officers and registration officers were to launch a special drive at once to enrol them.</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>ECI press release of 30.09.2026 (PIB)</t>
+          <t>ECI press note ECI/PN/120/2026 of 26.09.2026 | ECI press release of 26.09.2026 (PIB)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleasePage.aspx?PRID=2317352&amp;reg=3&amp;lang=1</t>
+          <t>https://www.eci.gov.in/eci/public/api/document?id=17536 | https://www.pib.gov.in/PressReleasePage.aspx?PRID=2315309&amp;reg=3&amp;lang=1</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -75226,57 +75226,94 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>The drive after the revision, in writing</t>
+          <t>Andhra Pradesh and Meghalaya extended</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>The Commission wrote to every Chief Electoral Officer setting out a special drive to enrol electors left off and young or first-time voters. Booth officers are to compare the current roll with the roll from before the revision, list everyone who was on the first and is missing from the second, visit them at home and help those found eligible fill in Form 6. The Commission asked them to cover at least 20 to 25 electors a week, so the work ends in about a month. The lists go to the booth agents of the recognised parties and then to the registration officer, who decides each case under the 1950 Act and the 1960 Rules. Booth camps are to be held, and special camps for people in night shelters, labour colonies and the homeless. The letter says anyone not on the roll, or whose name was deleted, can apply to be enrolled at any time.</t>
+          <t>Andhra Pradesh's notices run to 10 October and its final roll is due on 16 October 2026. Meghalaya's final roll moves to 26 October 2026.</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>ECI letter No. 23/2025/ERS(Vol-II) of 01.10.2026 to all Chief Electoral Officers</t>
+          <t>ECI press release of 30.09.2026 (PIB)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.eci.gov.in/eci/public/api/document?id=17541</t>
+          <t>https://www.pib.gov.in/PressReleasePage.aspx?PRID=2317352&amp;reg=3&amp;lang=1</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Election Commission</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Phase III</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>The drive after the revision, in writing</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>The Commission wrote to every Chief Electoral Officer setting out a special drive to enrol electors left off and young or first-time voters. Booth officers are to compare the current roll with the roll from before the revision, list everyone who was on the first and is missing from the second, visit them at home and help those found eligible fill in Form 6. The Commission asked them to cover at least 20 to 25 electors a week, so the work ends in about a month. The lists go to the booth agents of the recognised parties and then to the registration officer, who decides each case under the 1950 Act and the 1960 Rules. Booth camps are to be held, and special camps for people in night shelters, labour colonies and the homeless. The letter says anyone not on the roll, or whose name was deleted, can apply to be enrolled at any time.</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>ECI letter No. 23/2025/ERS(Vol-II) of 01.10.2026 to all Chief Electoral Officers</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>https://www.eci.gov.in/eci/public/api/document?id=17541</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>2026-10-03</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>State election officer</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>Phase III</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>A drive to find the names left off</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>When it published Uttarakhand's final roll, the state's Chief Electoral Officer set out the Commission's directions for what follows. Booth officers are to compare the roll from before the revision with the current one and list the electors who were on the first and are missing from the second. They are to visit them at home and help those still eligible fill in Form 6. The lists are to be shared with the booth agents of the recognised parties, and booth and special camps held, including for people in night shelters, labour colonies and the homeless.</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>CEO Uttarakhand, press note PN 63/2026 of 03.10.2026</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>https://cdnbbsr.s3waas.gov.in/s3cbf8710b43df3f2c1553e649403426df/uploads/2026/10/202610031173939115.pdf</t>
         </is>
@@ -79555,17 +79592,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Uttarakhand</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>7133785</v>
+        <v>9753577</v>
       </c>
       <c r="D4" t="n">
-        <v>2430000</v>
+        <v>3312919</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -79573,7 +79610,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>34.1</v>
+        <v>34</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -79582,53 +79619,56 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
-        </is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>1379785</v>
       </c>
       <c r="K4" t="n">
-        <v>1904380</v>
+        <v>1933134</v>
       </c>
       <c r="L4" t="n">
-        <v>97186</v>
+        <v>350</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>https://www.newindianexpress.com/india/2026/Aug/06/2027-lakh-voter-notices-trigger-political-row-in-uttarakhand-amid-electoral-roll-revision</t>
+          <t>https://www.hindustantimes.com/india-news/why-did-jaishankar-rekha-gupta-kejriwal-get-sir-notices-full-list-of-prominent-names-in-delhi-electoral-row-101789967719972.html</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>https://www.newindianexpress.com/india/2026/Aug/06/2027-lakh-voter-notices-trigger-political-row-in-uttarakhand-amid-electoral-roll-revision</t>
+          <t>https://www.hindustantimes.com/india-news/why-did-jaishankar-rekha-gupta-kejriwal-get-sir-notices-full-list-of-prominent-names-in-delhi-electoral-row-101789967719972.html</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>Tamil Nadu</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C5" t="n">
-        <v>9753577</v>
+        <v>54376756</v>
       </c>
       <c r="D5" t="n">
-        <v>3312919</v>
+        <v>17100000</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>published</t>
+          <t>sum</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>34</v>
+        <v>31.4</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -79637,56 +79677,56 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>1379785</v>
+        <v>1300000</v>
       </c>
       <c r="K5" t="n">
-        <v>1933134</v>
+        <v>15800000</v>
       </c>
       <c r="L5" t="n">
-        <v>350</v>
+        <v>2000</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>https://www.hindustantimes.com/india-news/why-did-jaishankar-rekha-gupta-kejriwal-get-sir-notices-full-list-of-prominent-names-in-delhi-electoral-row-101789967719972.html</t>
+          <t>https://www.newindianexpress.com/states/tamil-nadu/2026/Feb/24/electorate-shrinks-by-over-10-per-cent-in-tamil-nadus-103-constituencies</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>https://www.hindustantimes.com/india-news/why-did-jaishankar-rekha-gupta-kejriwal-get-sir-notices-full-list-of-prominent-names-in-delhi-electoral-row-101789967719972.html</t>
+          <t>https://www.newindianexpress.com/states/tamil-nadu/2026/Feb/24/electorate-shrinks-by-over-10-per-cent-in-tamil-nadus-103-constituencies</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tamil Nadu</t>
+          <t>Chandigarh</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C6" t="n">
-        <v>54376756</v>
+        <v>450282</v>
       </c>
       <c r="D6" t="n">
-        <v>17100000</v>
+        <v>137814</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>sum</t>
+          <t>published</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>31.4</v>
+        <v>30.6</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -79695,48 +79735,45 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>1300000</v>
+        <v>69461</v>
       </c>
       <c r="K6" t="n">
-        <v>15800000</v>
-      </c>
-      <c r="L6" t="n">
-        <v>2000</v>
+        <v>68353</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>https://www.newindianexpress.com/states/tamil-nadu/2026/Feb/24/electorate-shrinks-by-over-10-per-cent-in-tamil-nadus-103-constituencies</t>
+          <t>https://www.tribuneindia.com/news/chandigarh/sir-1-37-lakh-electors-to-get-notice-over-missing-linkage-discrepancies/</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>https://www.newindianexpress.com/states/tamil-nadu/2026/Feb/24/electorate-shrinks-by-over-10-per-cent-in-tamil-nadus-103-constituencies</t>
+          <t>https://www.tribuneindia.com/news/chandigarh/sir-1-37-lakh-electors-to-get-notice-over-missing-linkage-discrepancies/</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Chandigarh</t>
+          <t>Arunachal Pradesh</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>3</v>
       </c>
       <c r="C7" t="n">
-        <v>450282</v>
+        <v>718046</v>
       </c>
       <c r="D7" t="n">
-        <v>137814</v>
+        <v>218588</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -79744,11 +79781,11 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>30.6</v>
+        <v>30.4</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>press</t>
+          <t>primary</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -79758,40 +79795,43 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>69461</v>
+        <v>85175</v>
       </c>
       <c r="K7" t="n">
-        <v>68353</v>
+        <v>133413</v>
+      </c>
+      <c r="L7" t="n">
+        <v>28899</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>https://www.tribuneindia.com/news/chandigarh/sir-1-37-lakh-electors-to-get-notice-over-missing-linkage-discrepancies/</t>
+          <t>https://ceoarunachal.nic.in/componenthelper/getcomponentfile/68</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>https://www.tribuneindia.com/news/chandigarh/sir-1-37-lakh-electors-to-get-notice-over-missing-linkage-discrepancies/</t>
+          <t>https://ceoarunachal.nic.in/componenthelper/getcomponentfile/68</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Arunachal Pradesh</t>
+          <t>Meghalaya</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>3</v>
       </c>
       <c r="C8" t="n">
-        <v>718046</v>
+        <v>2169243</v>
       </c>
       <c r="D8" t="n">
-        <v>218588</v>
+        <v>651735</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -79799,11 +79839,11 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>30.4</v>
+        <v>30</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>primary</t>
+          <t>press</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -79813,43 +79853,43 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>85175</v>
+        <v>222786</v>
       </c>
       <c r="K8" t="n">
-        <v>133413</v>
+        <v>428949</v>
       </c>
       <c r="L8" t="n">
-        <v>28899</v>
+        <v>1194</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>https://ceoarunachal.nic.in/componenthelper/getcomponentfile/68</t>
+          <t>https://www.syllad.com/over-93-sir-notice-cases-resolved-blos-to-facilitate-electors-at-doorstep-meghalaya-ceo/</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>https://ceoarunachal.nic.in/componenthelper/getcomponentfile/68</t>
+          <t>https://www.syllad.com/over-93-sir-notice-cases-resolved-blos-to-facilitate-electors-at-doorstep-meghalaya-ceo/</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Meghalaya</t>
+          <t>Sikkim</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>3</v>
       </c>
       <c r="C9" t="n">
-        <v>2169243</v>
+        <v>433294</v>
       </c>
       <c r="D9" t="n">
-        <v>651735</v>
+        <v>124519</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -79857,11 +79897,11 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>30</v>
+        <v>28.7</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>press</t>
+          <t>primary</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -79871,43 +79911,43 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>222786</v>
+        <v>72135</v>
       </c>
       <c r="K9" t="n">
-        <v>428949</v>
+        <v>52384</v>
       </c>
       <c r="L9" t="n">
-        <v>1194</v>
+        <v>16485</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>https://www.syllad.com/over-93-sir-notice-cases-resolved-blos-to-facilitate-electors-at-doorstep-meghalaya-ceo/</t>
+          <t>https://www.sikkim.gov.in/media/news-announcement/news-info?name=Final+Electoral+Roll+under+SIR+2026+Published+in+Sikkim</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>https://www.syllad.com/over-93-sir-notice-cases-resolved-blos-to-facilitate-electors-at-doorstep-meghalaya-ceo/</t>
+          <t>https://www.sikkim.gov.in/media/news-announcement/news-info?name=Final+Electoral+Roll+under+SIR+2026+Published+in+Sikkim</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sikkim</t>
+          <t>Jharkhand</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>3</v>
       </c>
       <c r="C10" t="n">
-        <v>433294</v>
+        <v>22101249</v>
       </c>
       <c r="D10" t="n">
-        <v>124519</v>
+        <v>6324116</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -79915,11 +79955,11 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>28.7</v>
+        <v>28.6</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>primary</t>
+          <t>press</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -79929,43 +79969,35 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>72135</v>
+        <v>1403205</v>
       </c>
       <c r="K10" t="n">
-        <v>52384</v>
-      </c>
-      <c r="L10" t="n">
-        <v>16485</v>
+        <v>4555227</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>https://www.sikkim.gov.in/media/news-announcement/news-info?name=Final+Electoral+Roll+under+SIR+2026+Published+in+Sikkim</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>https://www.sikkim.gov.in/media/news-announcement/news-info?name=Final+Electoral+Roll+under+SIR+2026+Published+in+Sikkim</t>
+          <t>https://timesofindia.indiatimes.com/city/ranchi/jharkhand-electoral-roll-verification-notices-to-be-issued-to-63-24-lakh-voters/articleshow/133009630.cms</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Jharkhand</t>
+          <t>Uttarakhand</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>3</v>
       </c>
       <c r="C11" t="n">
-        <v>22101249</v>
+        <v>7133785</v>
       </c>
       <c r="D11" t="n">
-        <v>6324116</v>
+        <v>2027000</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -79973,7 +80005,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>28.6</v>
+        <v>28.4</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -79982,7 +80014,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -79990,15 +80022,20 @@
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="J11" t="n">
-        <v>1403205</v>
-      </c>
       <c r="K11" t="n">
-        <v>4555227</v>
+        <v>1904380</v>
+      </c>
+      <c r="L11" t="n">
+        <v>97186</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>https://timesofindia.indiatimes.com/city/ranchi/jharkhand-electoral-roll-verification-notices-to-be-issued-to-63-24-lakh-voters/articleshow/133009630.cms</t>
+          <t>https://www.newindianexpress.com/india/2026/Aug/06/2027-lakh-voter-notices-trigger-political-row-in-uttarakhand-amid-electoral-roll-revision</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>https://www.newindianexpress.com/india/2026/Aug/06/2027-lakh-voter-notices-trigger-political-row-in-uttarakhand-amid-electoral-roll-revision</t>
         </is>
       </c>
     </row>

</xml_diff>